<commit_message>
fix: resolve research score calculation in composite evaluator, expose 7 dimension scores in API schemas, and remove manual verify-from-CV phrasing from frontend
</commit_message>
<xml_diff>
--- a/data/analysis/collaboration_profiles.xlsx
+++ b/data/analysis/collaboration_profiles.xlsx
@@ -744,12 +744,12 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>[{"name": "Tayyaba Gul Tareen", "paper_count": 4}, {"name": "Jehanzeb Khan", "paper_count": 2}, {"name": "Muhammad Aamir", "paper_count": 2}]</t>
+          <t>[{"name": "Tayyaba Gul Tareen", "paper_count": 4}, {"name": "Muhammad Aamir", "paper_count": 2}, {"name": "Jehanzeb Khan", "paper_count": 2}]</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Candidate Tayyaba Gull has collaborated with 13 unique co-author(s) across 5 publication(s). They operate as a Medium-Group Researcher with an average of 4.6 authors per paper. The candidate has 3 recurring collaborator(s) (top co-authors: Tayyaba Gul Tareen (4 papers), Jehanzeb Khan (2 papers), Muhammad Aamir (2 papers)). Overall research collaboration network is categorized as Broad Network.</t>
+          <t>Candidate Tayyaba Gull has collaborated with 13 unique co-author(s) across 5 publication(s). They operate as a Medium-Group Researcher with an average of 4.6 authors per paper. The candidate has 3 recurring collaborator(s) (top co-authors: Tayyaba Gul Tareen (4 papers), Muhammad Aamir (2 papers), Jehanzeb Khan (2 papers)). Overall research collaboration network is categorized as Broad Network.</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -933,12 +933,12 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>[{"name": "S Tamoor Ul Hassan", "paper_count": 6}, {"name": "M Bennis", "paper_count": 4}, {"name": "M Latva Aho", "paper_count": 4}, {"name": "Ashraf", "paper_count": 2}, {"name": "S Samarakoon", "paper_count": 2}]</t>
+          <t>[{"name": "S Tamoor Ul Hassan", "paper_count": 6}, {"name": "M Latva Aho", "paper_count": 4}, {"name": "M Bennis", "paper_count": 4}, {"name": "Ashraf", "paper_count": 2}, {"name": "S Samarakoon", "paper_count": 2}]</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Candidate SYED TAMOORULHASSAN has collaborated with 18 unique co-author(s) across 7 publication(s). They operate as a Large-Group Researcher with an average of 5.6 authors per paper. The candidate has 6 recurring collaborator(s) (top co-authors: S Tamoor Ul Hassan (6 papers), M Bennis (4 papers), M Latva Aho (4 papers)). Overall research collaboration network is categorized as Broad Network.</t>
+          <t>Candidate SYED TAMOORULHASSAN has collaborated with 18 unique co-author(s) across 7 publication(s). They operate as a Large-Group Researcher with an average of 5.6 authors per paper. The candidate has 6 recurring collaborator(s) (top co-authors: S Tamoor Ul Hassan (6 papers), M Latva Aho (4 papers), M Bennis (4 papers)). Overall research collaboration network is categorized as Broad Network.</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -996,7 +996,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>[{"name": "Waheed Aftab Khan", "paper_count": 5}, {"name": "W A Khan", "paper_count": 4}, {"name": "G Abbas", "paper_count": 4}, {"name": "Hafiz Fuad Usman", "paper_count": 3}, {"name": "Ali Raza", "paper_count": 3}]</t>
+          <t>[{"name": "Waheed Aftab Khan", "paper_count": 5}, {"name": "W A Khan", "paper_count": 4}, {"name": "G Abbas", "paper_count": 4}, {"name": "Ali Raza", "paper_count": 3}, {"name": "Hafiz Fuad Usman", "paper_count": 3}]</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1122,12 +1122,12 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>[{"name": "Sheikh", "paper_count": 3}, {"name": "Shakil Rehman", "paper_count": 3}, {"name": "Noman Naseer", "paper_count": 3}, {"name": "Shakil R Sheikh", "paper_count": 3}, {"name": "Ghafoor", "paper_count": 2}]</t>
+          <t>[{"name": "Shakil Rehman", "paper_count": 3}, {"name": "Sheikh", "paper_count": 3}, {"name": "Shakil R Sheikh", "paper_count": 3}, {"name": "Noman Naseer", "paper_count": 3}, {"name": "Ghafoor", "paper_count": 2}]</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Candidate Muzzamil Ghaffar has collaborated with 23 unique co-author(s) across 6 publication(s). They operate as a Large-Group Researcher with an average of 6.7 authors per paper. The candidate has 7 recurring collaborator(s) (top co-authors: Sheikh (3 papers), Shakil Rehman (3 papers), Noman Naseer (3 papers)). Overall research collaboration network is categorized as Broad Network.</t>
+          <t>Candidate Muzzamil Ghaffar has collaborated with 23 unique co-author(s) across 6 publication(s). They operate as a Large-Group Researcher with an average of 6.7 authors per paper. The candidate has 7 recurring collaborator(s) (top co-authors: Shakil Rehman (3 papers), Sheikh (3 papers), Shakil R Sheikh (3 papers)). Overall research collaboration network is categorized as Broad Network.</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
@@ -1185,7 +1185,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>[{"name": "Zz Abidin", "paper_count": 5}, {"name": "Kamarudin", "paper_count": 4}, {"name": "Ayi Ashyap", "paper_count": 3}, {"name": "Ha Majid", "paper_count": 3}, {"name": "Mi Abbasi", "paper_count": 2}]</t>
+          <t>[{"name": "Zz Abidin", "paper_count": 5}, {"name": "Kamarudin", "paper_count": 4}, {"name": "Ayi Ashyap", "paper_count": 3}, {"name": "Ha Majid", "paper_count": 3}, {"name": "Mh Dahri", "paper_count": 2}]</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1248,12 +1248,12 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>[{"name": "Mihai Datcu", "paper_count": 10}, {"name": "Andrei Anghel", "paper_count": 10}, {"name": "Eleftheria Kalogirou", "paper_count": 3}, {"name": "Despina Makri", "paper_count": 2}, {"name": "M Tzouvaras", "paper_count": 2}]</t>
+          <t>[{"name": "Andrei Anghel", "paper_count": 10}, {"name": "Mihai Datcu", "paper_count": 10}, {"name": "Eleftheria Kalogirou", "paper_count": 3}, {"name": "Despina Makri", "paper_count": 2}, {"name": "E Kalogirou", "paper_count": 2}]</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Candidate Muhammad Amjad has collaborated with 23 unique co-author(s) across 16 publication(s). They operate as a Medium-Group Researcher with an average of 4.1 authors per paper. The candidate has 9 recurring collaborator(s) (top co-authors: Mihai Datcu (10 papers), Andrei Anghel (10 papers), Eleftheria Kalogirou (3 papers)). Overall research collaboration network is categorized as Broad Network.</t>
+          <t>Candidate Muhammad Amjad has collaborated with 23 unique co-author(s) across 16 publication(s). They operate as a Medium-Group Researcher with an average of 4.1 authors per paper. The candidate has 9 recurring collaborator(s) (top co-authors: Andrei Anghel (10 papers), Mihai Datcu (10 papers), Eleftheria Kalogirou (3 papers)). Overall research collaboration network is categorized as Broad Network.</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
@@ -1437,12 +1437,12 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>[{"name": "Claus Pahl", "paper_count": 5}, {"name": "Waheed Ur Rehman", "paper_count": 3}, {"name": "Nabil El Ioini", "paper_count": 3}, {"name": "Hamid R Barzegar", "paper_count": 3}, {"name": "Ibe Van Thillo", "paper_count": 2}]</t>
+          <t>[{"name": "Claus Pahl", "paper_count": 5}, {"name": "Waheed Ur Rehman", "paper_count": 3}, {"name": "Hamid R Barzegar", "paper_count": 3}, {"name": "Nabil El Ioini", "paper_count": 3}, {"name": "Ibe Van Thillo", "paper_count": 2}]</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>Candidate Zeeshan has collaborated with 26 unique co-author(s) across 10 publication(s). They operate as a Large-Group Researcher with an average of 5.2 authors per paper. The candidate has 6 recurring collaborator(s) (top co-authors: Claus Pahl (5 papers), Waheed Ur Rehman (3 papers), Nabil El Ioini (3 papers)). Overall research collaboration network is categorized as Broad Network.</t>
+          <t>Candidate Zeeshan has collaborated with 26 unique co-author(s) across 10 publication(s). They operate as a Large-Group Researcher with an average of 5.2 authors per paper. The candidate has 6 recurring collaborator(s) (top co-authors: Claus Pahl (5 papers), Waheed Ur Rehman (3 papers), Hamid R Barzegar (3 papers)). Overall research collaboration network is categorized as Broad Network.</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
@@ -1500,12 +1500,12 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>[{"name": "Muhammad Saadi", "paper_count": 7}, {"name": "Jun Bae Seo", "paper_count": 6}, {"name": "Hu Jin", "paper_count": 6}, {"name": "Lunchakorn Wuttisittikulkij", "paper_count": 3}, {"name": "Naeem Maroof", "paper_count": 3}]</t>
+          <t>[{"name": "Muhammad Saadi", "paper_count": 7}, {"name": "Hu Jin", "paper_count": 6}, {"name": "Jun Bae Seo", "paper_count": 6}, {"name": "Lunchakorn Wuttisittikulkij", "paper_count": 3}, {"name": "Saqib Ali Khan", "paper_count": 3}]</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>Candidate Waqas Tariq Toor has collaborated with 83 unique co-author(s) across 29 publication(s). They operate as a Large-Group Researcher with an average of 5.1 authors per paper. The candidate has 15 recurring collaborator(s) (top co-authors: Muhammad Saadi (7 papers), Jun Bae Seo (6 papers), Hu Jin (6 papers)). Overall research collaboration network is categorized as Broad Network.</t>
+          <t>Candidate Waqas Tariq Toor has collaborated with 83 unique co-author(s) across 29 publication(s). They operate as a Large-Group Researcher with an average of 5.1 authors per paper. The candidate has 15 recurring collaborator(s) (top co-authors: Muhammad Saadi (7 papers), Hu Jin (6 papers), Jun Bae Seo (6 papers)). Overall research collaboration network is categorized as Broad Network.</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
@@ -1626,7 +1626,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>[{"name": "Danish Khan", "paper_count": 7}, {"name": "Manoj Kumar Panjwani", "paper_count": 4}, {"name": "Tahir Iqbal", "paper_count": 3}, {"name": "Honglu Zhu", "paper_count": 3}, {"name": "Qiang Lu", "paper_count": 2}]</t>
+          <t>[{"name": "Danish Khan", "paper_count": 7}, {"name": "Manoj Kumar Panjwani", "paper_count": 4}, {"name": "Tahir Iqbal", "paper_count": 3}, {"name": "Honglu Zhu", "paper_count": 3}, {"name": "Chang Qing Dong", "paper_count": 2}]</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -1752,7 +1752,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>[{"name": "F S", "paper_count": 9}, {"name": "M", "paper_count": 6}, {"name": "Sugiyama", "paper_count": 5}, {"name": "Y", "paper_count": 5}, {"name": "K", "paper_count": 5}]</t>
+          <t>[{"name": "F S", "paper_count": 9}, {"name": "M", "paper_count": 6}, {"name": "Sugiyama", "paper_count": 5}, {"name": "K", "paper_count": 5}, {"name": "Fujii", "paper_count": 5}]</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -2382,12 +2382,12 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>[{"name": "Sobia Jangsher", "paper_count": 4}, {"name": "Adnan Zafar", "paper_count": 2}, {"name": "Ashfaq Ahmed", "paper_count": 2}]</t>
+          <t>[{"name": "Sobia Jangsher", "paper_count": 4}, {"name": "Ashfaq Ahmed", "paper_count": 2}, {"name": "Adnan Zafar", "paper_count": 2}]</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>Candidate Aamina Akbar has collaborated with 7 unique co-author(s) across 4 publication(s). They operate as a Medium-Group Researcher with an average of 4.0 authors per paper. The candidate has 3 recurring collaborator(s) (top co-authors: Sobia Jangsher (4 papers), Adnan Zafar (2 papers), Ashfaq Ahmed (2 papers)). Overall research collaboration network is categorized as Balanced Network.</t>
+          <t>Candidate Aamina Akbar has collaborated with 7 unique co-author(s) across 4 publication(s). They operate as a Medium-Group Researcher with an average of 4.0 authors per paper. The candidate has 3 recurring collaborator(s) (top co-authors: Sobia Jangsher (4 papers), Ashfaq Ahmed (2 papers), Adnan Zafar (2 papers)). Overall research collaboration network is categorized as Balanced Network.</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
@@ -2445,12 +2445,12 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>[{"name": "Syed Ali Hassan", "paper_count": 7}, {"name": "Shah Zeb", "paper_count": 4}, {"name": "Aamir Mahmood", "paper_count": 2}, {"name": "Mikael Gidlund", "paper_count": 2}, {"name": "Syed Ali Raza Zaidi", "paper_count": 2}]</t>
+          <t>[{"name": "Syed Ali Hassan", "paper_count": 7}, {"name": "Shah Zeb", "paper_count": 4}, {"name": "Mikael Gidlund", "paper_count": 2}, {"name": "Aamir Mahmood", "paper_count": 2}, {"name": "Syed Ali Raza Zaidi", "paper_count": 2}]</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>Candidate Qamar Abbas has collaborated with 12 unique co-author(s) across 7 publication(s). They operate as a Medium-Group Researcher with an average of 4.7 authors per paper. The candidate has 7 recurring collaborator(s) (top co-authors: Syed Ali Hassan (7 papers), Shah Zeb (4 papers), Aamir Mahmood (2 papers)). Overall research collaboration network is categorized as Balanced Network.</t>
+          <t>Candidate Qamar Abbas has collaborated with 12 unique co-author(s) across 7 publication(s). They operate as a Medium-Group Researcher with an average of 4.7 authors per paper. The candidate has 7 recurring collaborator(s) (top co-authors: Syed Ali Hassan (7 papers), Shah Zeb (4 papers), Mikael Gidlund (2 papers)). Overall research collaboration network is categorized as Balanced Network.</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
@@ -2508,12 +2508,12 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>[{"name": "Eun Sung Jung", "paper_count": 5}, {"name": "Hyung Seok Kim", "paper_count": 5}, {"name": "Amir Haider", "paper_count": 4}, {"name": "Rashid Ali", "paper_count": 4}, {"name": "M Zubair Islam", "paper_count": 2}]</t>
+          <t>[{"name": "Eun Sung Jung", "paper_count": 5}, {"name": "Hyung Seok Kim", "paper_count": 5}, {"name": "Rashid Ali", "paper_count": 4}, {"name": "Amir Haider", "paper_count": 4}, {"name": "M Zubair Islam", "paper_count": 2}]</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>Candidate Shahzad has collaborated with 8 unique co-author(s) across 9 publication(s). They operate as a Medium-Group Researcher with an average of 3.6 authors per paper. The candidate has 5 recurring collaborator(s) (top co-authors: Eun Sung Jung (5 papers), Hyung Seok Kim (5 papers), Amir Haider (4 papers)). Overall research collaboration network is categorized as Balanced Network.</t>
+          <t>Candidate Shahzad has collaborated with 8 unique co-author(s) across 9 publication(s). They operate as a Medium-Group Researcher with an average of 3.6 authors per paper. The candidate has 5 recurring collaborator(s) (top co-authors: Eun Sung Jung (5 papers), Hyung Seok Kim (5 papers), Rashid Ali (4 papers)). Overall research collaboration network is categorized as Balanced Network.</t>
         </is>
       </c>
       <c r="O33" t="inlineStr">
@@ -3348,7 +3348,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Fazal Muhammad</t>
+          <t>Shanshan Tu</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -3369,7 +3369,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Ammar Armghan</t>
+          <t>Asar Ali</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -3390,7 +3390,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Asar Ali</t>
+          <t>Ammar Armghan</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -3453,7 +3453,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Shanshan Tu</t>
+          <t>Fazal Muhammad</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -3537,7 +3537,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Salman A Alqahtani</t>
+          <t>Amil Daraz</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -3558,7 +3558,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Amil Daraz</t>
+          <t>Atif M Alamri</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -3579,7 +3579,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Atif M Alamri</t>
+          <t>Salman A Alqahtani</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -3663,7 +3663,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Salman Ahmed</t>
+          <t>Ghulam E Mustafa Abro</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -3684,7 +3684,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Abdul Rehman Altaf</t>
+          <t>Salman Ahmed</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3705,7 +3705,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Abdinasir Hirsi</t>
+          <t>Ardhi Wijayanto</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3726,7 +3726,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Nabihah Ahmad</t>
+          <t>Abdinasir Hirsi</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3747,7 +3747,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Ghulam E Mustafa Abro</t>
+          <t>Nabihah Ahmad</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3768,7 +3768,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Ardhi Wijayanto</t>
+          <t>Abdul Rehman Altaf</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3789,7 +3789,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Achraf Jabeur Telmoudi</t>
+          <t>Syed Tahir Hussain Rizvi</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3810,7 +3810,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Muhammad Yasir Latif</t>
+          <t>Muhammad Saad Amin</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3831,7 +3831,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Muhammad Saad Amin</t>
+          <t>Achraf Jabeur Telmoudi</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3852,7 +3852,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Syed Tahir Hussain Rizvi</t>
+          <t>Muhammad Yasir Latif</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -3999,7 +3999,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Daoliang Li</t>
+          <t>Usama Iqbal</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4020,7 +4020,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Usama Iqbal</t>
+          <t>Daoliang Li</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -4209,7 +4209,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Rahmat Ullah</t>
+          <t>Syeda Javeria Ahsan</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -4272,7 +4272,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Syeda Javeria Ahsan</t>
+          <t>Rahmat Ullah</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -4314,7 +4314,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Yan Xu</t>
+          <t>Arsalan Khurshid</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -4335,7 +4335,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Wei Chen</t>
+          <t>Saadullah Farooq Abbasi</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -4356,7 +4356,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Chen Chen</t>
+          <t>Yan Xu</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -4377,7 +4377,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Arsalan Khurshid</t>
+          <t>Chen Chen</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -4398,7 +4398,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Saadullah Farooq Abbasi</t>
+          <t>Wei Chen</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -4419,7 +4419,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Laishuan Wang</t>
+          <t>Hafza Ayesha Siddiqa</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -4440,7 +4440,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Hafza Ayesha Siddiqa</t>
+          <t>Laishuan Wang</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -4524,7 +4524,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Mohammad Qasim Shahid</t>
+          <t>Ali Imran</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -4545,7 +4545,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Ali Imran</t>
+          <t>Hussain Al Faisal</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -4566,7 +4566,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Hussain Al Faisal</t>
+          <t>Mohammad Qasim Shahid</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -4755,7 +4755,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Sabtain Raza</t>
+          <t>Aqeel Ahmed Khan</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -4776,7 +4776,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Muhammad Taha</t>
+          <t>Sabtain Raza</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -4797,7 +4797,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Aqeel Ahmed Khan</t>
+          <t>Muhammad Taha</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -4818,7 +4818,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Anzar Mahmood</t>
+          <t>Qamar Akhter</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -4860,7 +4860,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Waseem Aslam</t>
+          <t>Salman A Alqahtani</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -4881,7 +4881,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Salman A Alqahtani</t>
+          <t>Paranav Kumar Pathak</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -4902,7 +4902,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Qamar Akhter</t>
+          <t>Mehboob Alam</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -4923,7 +4923,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Paranav Kumar Pathak</t>
+          <t>Waseem Aslam</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -4944,7 +4944,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Mehboob Alam</t>
+          <t>Anzar Mahmood</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -4986,7 +4986,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Ahsan Shahzad</t>
+          <t>Yazeed Yasin Ghadi</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -5007,7 +5007,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Faisal Jamil</t>
+          <t>Ahsan Shahzad</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -5028,7 +5028,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Yazeed Yasin Ghadi</t>
+          <t>Faisal Jamil</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -5070,7 +5070,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Khalid Alhussaini</t>
+          <t>Uroosa Nawaz</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -5091,7 +5091,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Uroosa Nawaz</t>
+          <t>Khalid Alhussaini</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -5112,7 +5112,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Adham Aleid</t>
+          <t>Saman Khalil</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -5154,7 +5154,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Saman Khalil</t>
+          <t>Adham Aleid</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -5196,7 +5196,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Noor Afshan</t>
+          <t>Imran Siddique</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -5217,7 +5217,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Nabeel Ahmed Khan</t>
+          <t>Noor Afshan</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -5238,7 +5238,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Imran Siddique</t>
+          <t>Nabeel Ahmed Khan</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -5343,7 +5343,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Olivier D</t>
+          <t>Arsalan Habib</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -5364,7 +5364,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Usman</t>
+          <t>Khawaja</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -5385,7 +5385,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Saqib</t>
+          <t>Bernal</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -5406,7 +5406,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Arsalan Habib</t>
+          <t>Usman</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -5448,7 +5448,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Zabit</t>
+          <t>Bosch</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -5469,7 +5469,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Khawaja</t>
+          <t>Amin</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -5490,7 +5490,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Saqib</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -5511,7 +5511,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Amin</t>
+          <t>Zabit</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -5532,7 +5532,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Bernal</t>
+          <t>Olivier D</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -5553,7 +5553,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Shehla</t>
+          <t>Inam</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -5574,7 +5574,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Muhammad Ziaur</t>
+          <t>Rehman</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -5595,7 +5595,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Inam</t>
+          <t>Muhammad Ziaur</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -5616,7 +5616,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Rehman</t>
+          <t>Shehla</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -5952,7 +5952,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Jehanzeb Khan</t>
+          <t>Muhammad Aamir</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -5973,7 +5973,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Muhammad Aamir</t>
+          <t>Jehanzeb Khan</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -6057,7 +6057,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Shahryar Shafique</t>
+          <t>Mehr E Munir</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -6078,7 +6078,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Mehr E Munir</t>
+          <t>Shahryar Shafique</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -6099,7 +6099,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Nasir Saleem</t>
+          <t>Tayyaba Tareen</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -6120,7 +6120,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Sher Ali</t>
+          <t>Nasir Saleem</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -6141,7 +6141,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Tayyaba Tareen</t>
+          <t>Sher Ali</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -6162,7 +6162,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>Fakhar Anjam</t>
+          <t>Ghassan Husnain</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -6183,7 +6183,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>Ghassan Husnain</t>
+          <t>Fakhar Anjam</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -6330,7 +6330,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>Muhammad Faheem</t>
+          <t>Khalid Masood</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -6351,7 +6351,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Khalid Masood</t>
+          <t>Muhammad Faheem</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -6372,7 +6372,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>Khalil Ur Rehman</t>
+          <t>Bo Wang</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -6393,7 +6393,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>Bo Wang</t>
+          <t>Khalil Ur Rehman</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -6477,7 +6477,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>Farman Ali</t>
+          <t>Shoaib U</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -6498,7 +6498,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>Shoaib U</t>
+          <t>Farman Ali</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -6519,7 +6519,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>Muhammad Haseeb Zia</t>
+          <t>Khola Farooq</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -6540,7 +6540,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>Khola Farooq</t>
+          <t>Muhammad Haseeb Zia</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -6561,7 +6561,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>Faiza Rehman</t>
+          <t>Saima Yousaf</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -6582,7 +6582,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>Shoaib Saleem</t>
+          <t>Faiza Rehman</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -6603,7 +6603,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>Saima Yousaf</t>
+          <t>Shoaib Saleem</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -6624,7 +6624,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>Hadi Abdullah</t>
+          <t>Saba Mohsin</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -6645,7 +6645,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>Syeda Urwa Warsi</t>
+          <t>Hadi Abdullah</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -6666,7 +6666,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>Saba Mohsin</t>
+          <t>Syeda Urwa Warsi</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -6729,7 +6729,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>Amber Sultan</t>
+          <t>Junaid Waseem</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -6750,7 +6750,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>Hanan Sharif</t>
+          <t>Amber Sultan</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -6771,7 +6771,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>Junaid Waseem</t>
+          <t>Hanan Sharif</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -6834,7 +6834,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>Muhammad Sohail</t>
+          <t>Muhammad Arfan Ali Nagra</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -6855,7 +6855,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>Muhammad Mudassar</t>
+          <t>Muhammad Sohail</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -6876,7 +6876,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>Muhammad Arfan Ali Nagra</t>
+          <t>Muhammad Mudassar</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -6918,7 +6918,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>Alghamdi</t>
+          <t>Sultan H Almotiri</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -6960,7 +6960,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>Sultan H Almotiri</t>
+          <t>Alghamdi</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -6981,7 +6981,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>Anas Bilal</t>
+          <t>Ahmad Alshammari</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -7023,7 +7023,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>Muhammad Ahsan Raza</t>
+          <t>Anas Bilal</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -7044,7 +7044,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>Ahmad Alshammari</t>
+          <t>Muhammad Ahsan Raza</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -7065,7 +7065,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>Saifur Rahman Khan</t>
+          <t>Muhammad Irfan</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -7086,7 +7086,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>Tomasz Jakubowski</t>
+          <t>Nabeel Ahmed</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -7107,7 +7107,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>Zohaib Mushtaq</t>
+          <t>Paweł Sokołowski</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -7128,7 +7128,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>Muhammad Irfan</t>
+          <t>Zohaib Mushtaq</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -7149,7 +7149,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>Grzegorz Nawalany</t>
+          <t>Tomasz Jakubowski</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -7170,7 +7170,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>Paweł Sokołowski</t>
+          <t>Grzegorz Nawalany</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -7191,7 +7191,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>Nabeel Ahmed</t>
+          <t>Saifur Rahman Khan</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -7275,7 +7275,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>Kashif</t>
+          <t>Ameer</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -7296,7 +7296,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>Saqib Ameer</t>
+          <t>Kashif</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -7338,7 +7338,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>Ameer</t>
+          <t>Saqib Ameer</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -7359,7 +7359,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>Hussain</t>
+          <t>Xiang Lin Zhu</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -7380,7 +7380,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>Muhammad Ajmal</t>
+          <t>Hussain</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -7401,7 +7401,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>Xiang Lin Zhu</t>
+          <t>Muhammad Ajmal</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -7422,7 +7422,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>Talal Ahmad</t>
+          <t>Noor Rehman</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -7443,7 +7443,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>Noor Rehman</t>
+          <t>Muhammad Saeed</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -7464,7 +7464,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>Muhammad Saeed</t>
+          <t>Talal Ahmad</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -7485,7 +7485,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>Benjamin Doh</t>
+          <t>Benjamin Kwame Adobah</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -7506,7 +7506,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>Benjamin Kwame Adobah</t>
+          <t>Benjamin Doh</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -7548,7 +7548,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>Han F</t>
+          <t>Ling Qh</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -7569,7 +7569,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>Ling Qh</t>
+          <t>Mehta S</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -7590,7 +7590,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>Mehta S</t>
+          <t>Han F</t>
         </is>
       </c>
       <c r="C208" t="n">
@@ -7674,7 +7674,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>Sheikh Junaid Yawar</t>
+          <t>Haris Jawad Arain</t>
         </is>
       </c>
       <c r="C212" t="n">
@@ -7695,7 +7695,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>Haris Jawad Arain</t>
+          <t>Sheikh Junaid Yawar</t>
         </is>
       </c>
       <c r="C213" t="n">
@@ -7989,7 +7989,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>Abdullah Amankhan</t>
+          <t>Khalidumer</t>
         </is>
       </c>
       <c r="C227" t="n">
@@ -8010,7 +8010,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>Khalidumer</t>
+          <t>Abdullah Amankhan</t>
         </is>
       </c>
       <c r="C228" t="n">
@@ -8325,7 +8325,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>A Raza</t>
+          <t>M Naeem</t>
         </is>
       </c>
       <c r="C243" t="n">
@@ -8346,7 +8346,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>M Naeem</t>
+          <t>A Raza</t>
         </is>
       </c>
       <c r="C244" t="n">
@@ -8493,7 +8493,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>Dongsheng Cai</t>
+          <t>Ateeq</t>
         </is>
       </c>
       <c r="C251" t="n">
@@ -8514,7 +8514,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>Ateeq</t>
+          <t>Dongsheng Cai</t>
         </is>
       </c>
       <c r="C252" t="n">
@@ -8556,7 +8556,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>Rajesh Kumar</t>
+          <t>Sidra Sha(cid:0)q</t>
         </is>
       </c>
       <c r="C254" t="n">
@@ -8598,7 +8598,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>Sidra Sha(cid:0)q</t>
+          <t>Rajesh Kumar</t>
         </is>
       </c>
       <c r="C256" t="n">
@@ -8619,7 +8619,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>Nermish Mushtaq</t>
+          <t>Iqra Nazir</t>
         </is>
       </c>
       <c r="C257" t="n">
@@ -8640,7 +8640,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>Iqra Nazir</t>
+          <t>Nermish Mushtaq</t>
         </is>
       </c>
       <c r="C258" t="n">
@@ -8661,7 +8661,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>Sania Kanwal</t>
+          <t>Sadeed Ahmad</t>
         </is>
       </c>
       <c r="C259" t="n">
@@ -8682,7 +8682,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>Sadeed Ahmad</t>
+          <t>Sania Kanwal</t>
         </is>
       </c>
       <c r="C260" t="n">
@@ -8724,7 +8724,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>Bilal Ra(cid:0)que</t>
+          <t>Iqra Batool</t>
         </is>
       </c>
       <c r="C262" t="n">
@@ -8745,7 +8745,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>Iqra Batool</t>
+          <t>Bilal Ra(cid:0)que</t>
         </is>
       </c>
       <c r="C263" t="n">
@@ -8787,7 +8787,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>Sarathbabu</t>
+          <t>Kola Narasimha</t>
         </is>
       </c>
       <c r="C265" t="n">
@@ -8808,7 +8808,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>Raju</t>
+          <t>Sarathbabu</t>
         </is>
       </c>
       <c r="C266" t="n">
@@ -8829,7 +8829,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>Kola Narasimha</t>
+          <t>Raju</t>
         </is>
       </c>
       <c r="C267" t="n">
@@ -8871,7 +8871,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>Syed Adrees Ahmad</t>
+          <t>Asif Raza</t>
         </is>
       </c>
       <c r="C269" t="n">
@@ -8892,7 +8892,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>Asif Raza</t>
+          <t>Syed Adrees Ahmad</t>
         </is>
       </c>
       <c r="C270" t="n">
@@ -9039,7 +9039,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>M Bennis</t>
+          <t>M Latva Aho</t>
         </is>
       </c>
       <c r="C277" t="n">
@@ -9060,7 +9060,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>M Latva Aho</t>
+          <t>M Bennis</t>
         </is>
       </c>
       <c r="C278" t="n">
@@ -9165,7 +9165,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>H Chowdhury</t>
+          <t>M Ikram</t>
         </is>
       </c>
       <c r="C283" t="n">
@@ -9186,7 +9186,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>Marcos Katz</t>
+          <t>H Chowdhury</t>
         </is>
       </c>
       <c r="C284" t="n">
@@ -9207,7 +9207,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>M Ikram</t>
+          <t>Marcos Katz</t>
         </is>
       </c>
       <c r="C285" t="n">
@@ -9228,7 +9228,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>Kim Fung Tsang</t>
+          <t>Jonathan Rodriquez</t>
         </is>
       </c>
       <c r="C286" t="n">
@@ -9249,7 +9249,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>Muhammad Ikram</t>
+          <t>Syed Tamoor Ul Hassan</t>
         </is>
       </c>
       <c r="C287" t="n">
@@ -9270,7 +9270,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>Syed Tamoor Ul Hassan</t>
+          <t>Kim Fung Tsang</t>
         </is>
       </c>
       <c r="C288" t="n">
@@ -9291,7 +9291,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>Jonathan Rodriquez</t>
+          <t>Muhammad Ikram</t>
         </is>
       </c>
       <c r="C289" t="n">
@@ -9459,7 +9459,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>Hafiz Fuad Usman</t>
+          <t>Ali Raza</t>
         </is>
       </c>
       <c r="C297" t="n">
@@ -9480,7 +9480,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>Ali Raza</t>
+          <t>Hafiz Fuad Usman</t>
         </is>
       </c>
       <c r="C298" t="n">
@@ -9753,7 +9753,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Muhammad Rehan Usman</t>
+          <t>Waheed A Khan</t>
         </is>
       </c>
       <c r="C311" t="n">
@@ -9795,7 +9795,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Kamran Daniel</t>
+          <t>Muhammad Rehan Usman</t>
         </is>
       </c>
       <c r="C313" t="n">
@@ -9816,7 +9816,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Waheed A Khan</t>
+          <t>Kamran Daniel</t>
         </is>
       </c>
       <c r="C314" t="n">
@@ -9858,7 +9858,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Heba G Mohamed</t>
+          <t>Nouman Ali</t>
         </is>
       </c>
       <c r="C316" t="n">
@@ -9879,7 +9879,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Zhassulan Orazbekov</t>
+          <t>Muhammad Ilyas Menhas</t>
         </is>
       </c>
       <c r="C317" t="n">
@@ -9900,7 +9900,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Faisal Mehmood Butt</t>
+          <t>Heba G Mohamed</t>
         </is>
       </c>
       <c r="C318" t="n">
@@ -9921,7 +9921,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Nouman Ali</t>
+          <t>Sohaib Manzoor</t>
         </is>
       </c>
       <c r="C319" t="n">
@@ -9942,7 +9942,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Muhammad Ilyas Menhas</t>
+          <t>Zhassulan Orazbekov</t>
         </is>
       </c>
       <c r="C320" t="n">
@@ -9963,7 +9963,7 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Umair Ahmad Salaria</t>
+          <t>Faisal Mehmood Butt</t>
         </is>
       </c>
       <c r="C321" t="n">
@@ -9984,7 +9984,7 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Sohaib Manzoor</t>
+          <t>Umair Ahmad Salaria</t>
         </is>
       </c>
       <c r="C322" t="n">
@@ -10005,7 +10005,7 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Wajih H Hashmi</t>
+          <t>Tahir Zaidi</t>
         </is>
       </c>
       <c r="C323" t="n">
@@ -10047,7 +10047,7 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>Tahir Zaidi</t>
+          <t>Wajih H Hashmi</t>
         </is>
       </c>
       <c r="C325" t="n">
@@ -10068,7 +10068,7 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>Qaiser Nadeem</t>
+          <t>Jannat Bakht</t>
         </is>
       </c>
       <c r="C326" t="n">
@@ -10089,7 +10089,7 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>Shafaqut Ali</t>
+          <t>Qaiser Nadeem</t>
         </is>
       </c>
       <c r="C327" t="n">
@@ -10110,7 +10110,7 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>Jannat Bakht</t>
+          <t>Shafaqut Ali</t>
         </is>
       </c>
       <c r="C328" t="n">
@@ -10152,7 +10152,7 @@
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>Daesik Jeong</t>
+          <t>Arslan Usman</t>
         </is>
       </c>
       <c r="C330" t="n">
@@ -10173,7 +10173,7 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>Rizwan Ali Naqvi</t>
+          <t>Seung Won Lee</t>
         </is>
       </c>
       <c r="C331" t="n">
@@ -10194,7 +10194,7 @@
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>Hammad Riaz</t>
+          <t>Daesik Jeong</t>
         </is>
       </c>
       <c r="C332" t="n">
@@ -10215,7 +10215,7 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>M Rehan Usman</t>
+          <t>Hammad Riaz</t>
         </is>
       </c>
       <c r="C333" t="n">
@@ -10236,7 +10236,7 @@
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>Seung Won Lee</t>
+          <t>M Rehan Usman</t>
         </is>
       </c>
       <c r="C334" t="n">
@@ -10257,7 +10257,7 @@
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>Arslan Usman</t>
+          <t>Rizwan Ali Naqvi</t>
         </is>
       </c>
       <c r="C335" t="n">
@@ -10278,7 +10278,7 @@
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Wah Hoon Siew</t>
+          <t>Zixin Guo</t>
         </is>
       </c>
       <c r="C336" t="n">
@@ -10320,7 +10320,7 @@
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>Zixin Guo</t>
+          <t>Wah Hoon Siew</t>
         </is>
       </c>
       <c r="C338" t="n">
@@ -10362,7 +10362,7 @@
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>Talha Gul</t>
+          <t>Umar Saleem</t>
         </is>
       </c>
       <c r="C340" t="n">
@@ -10383,7 +10383,7 @@
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>Umar Saleem</t>
+          <t>Usman Arshad</t>
         </is>
       </c>
       <c r="C341" t="n">
@@ -10404,7 +10404,7 @@
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>Usman Arshad</t>
+          <t>Talha Gul</t>
         </is>
       </c>
       <c r="C342" t="n">
@@ -10425,7 +10425,7 @@
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>Sm Ali</t>
+          <t>Z Ullah</t>
         </is>
       </c>
       <c r="C343" t="n">
@@ -10467,7 +10467,7 @@
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>Z Ullah</t>
+          <t>F Wahab</t>
         </is>
       </c>
       <c r="C345" t="n">
@@ -10488,7 +10488,7 @@
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>F Wahab</t>
+          <t>Sm Ali</t>
         </is>
       </c>
       <c r="C346" t="n">
@@ -10551,7 +10551,7 @@
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>S Hamid</t>
+          <t>H F Usman</t>
         </is>
       </c>
       <c r="C349" t="n">
@@ -10572,7 +10572,7 @@
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>A Yousaf</t>
+          <t>S Hamid</t>
         </is>
       </c>
       <c r="C350" t="n">
@@ -10593,7 +10593,7 @@
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>H F Usman</t>
+          <t>A Yousaf</t>
         </is>
       </c>
       <c r="C351" t="n">
@@ -10614,7 +10614,7 @@
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>S Kaleem</t>
+          <t>H Farooq</t>
         </is>
       </c>
       <c r="C352" t="n">
@@ -10677,7 +10677,7 @@
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>H Farooq</t>
+          <t>S Kaleem</t>
         </is>
       </c>
       <c r="C355" t="n">
@@ -10740,7 +10740,7 @@
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>M Usman</t>
+          <t>M T Gul</t>
         </is>
       </c>
       <c r="C358" t="n">
@@ -10761,7 +10761,7 @@
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>M T Gul</t>
+          <t>M Usman</t>
         </is>
       </c>
       <c r="C359" t="n">
@@ -10887,7 +10887,7 @@
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>J Gu</t>
+          <t>G B Satrya</t>
         </is>
       </c>
       <c r="C365" t="n">
@@ -10929,7 +10929,7 @@
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>G B Satrya</t>
+          <t>J Gu</t>
         </is>
       </c>
       <c r="C367" t="n">
@@ -11076,7 +11076,7 @@
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t>M Brunero</t>
+          <t>L Potì</t>
         </is>
       </c>
       <c r="C374" t="n">
@@ -11097,7 +11097,7 @@
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>M Ferrari</t>
+          <t>P Nadimi Goki</t>
         </is>
       </c>
       <c r="C375" t="n">
@@ -11118,7 +11118,7 @@
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>E Paolini</t>
+          <t>N Andriolli</t>
         </is>
       </c>
       <c r="C376" t="n">
@@ -11139,7 +11139,7 @@
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t>L Potì</t>
+          <t>A Gatto</t>
         </is>
       </c>
       <c r="C377" t="n">
@@ -11160,7 +11160,7 @@
       </c>
       <c r="B378" t="inlineStr">
         <is>
-          <t>P Nadimi Goki</t>
+          <t>M Brunero</t>
         </is>
       </c>
       <c r="C378" t="n">
@@ -11181,7 +11181,7 @@
       </c>
       <c r="B379" t="inlineStr">
         <is>
-          <t>A Gatto</t>
+          <t>S Civelli</t>
         </is>
       </c>
       <c r="C379" t="n">
@@ -11202,7 +11202,7 @@
       </c>
       <c r="B380" t="inlineStr">
         <is>
-          <t>S Civelli</t>
+          <t>M Ferrari</t>
         </is>
       </c>
       <c r="C380" t="n">
@@ -11223,7 +11223,7 @@
       </c>
       <c r="B381" t="inlineStr">
         <is>
-          <t>N Andriolli</t>
+          <t>E Paolini</t>
         </is>
       </c>
       <c r="C381" t="n">
@@ -11391,7 +11391,7 @@
       </c>
       <c r="B389" t="inlineStr">
         <is>
-          <t>Sheikh</t>
+          <t>Shakil Rehman</t>
         </is>
       </c>
       <c r="C389" t="n">
@@ -11412,7 +11412,7 @@
       </c>
       <c r="B390" t="inlineStr">
         <is>
-          <t>Shakil Rehman</t>
+          <t>Sheikh</t>
         </is>
       </c>
       <c r="C390" t="n">
@@ -11433,7 +11433,7 @@
       </c>
       <c r="B391" t="inlineStr">
         <is>
-          <t>Noman Naseer</t>
+          <t>Shakil R Sheikh</t>
         </is>
       </c>
       <c r="C391" t="n">
@@ -11454,7 +11454,7 @@
       </c>
       <c r="B392" t="inlineStr">
         <is>
-          <t>Shakil R Sheikh</t>
+          <t>Noman Naseer</t>
         </is>
       </c>
       <c r="C392" t="n">
@@ -11538,7 +11538,7 @@
       </c>
       <c r="B396" t="inlineStr">
         <is>
-          <t>Noman</t>
+          <t>Bashir Salah</t>
         </is>
       </c>
       <c r="C396" t="n">
@@ -11559,7 +11559,7 @@
       </c>
       <c r="B397" t="inlineStr">
         <is>
-          <t>Bashir Salah</t>
+          <t>Soliman Alkhatib</t>
         </is>
       </c>
       <c r="C397" t="n">
@@ -11580,7 +11580,7 @@
       </c>
       <c r="B398" t="inlineStr">
         <is>
-          <t>Soliman Alkhatib</t>
+          <t>Naseer</t>
         </is>
       </c>
       <c r="C398" t="n">
@@ -11601,7 +11601,7 @@
       </c>
       <c r="B399" t="inlineStr">
         <is>
-          <t>Naseer</t>
+          <t>Noman</t>
         </is>
       </c>
       <c r="C399" t="n">
@@ -11685,7 +11685,7 @@
       </c>
       <c r="B403" t="inlineStr">
         <is>
-          <t>Koreshi</t>
+          <t>Muhammad</t>
         </is>
       </c>
       <c r="C403" t="n">
@@ -11706,7 +11706,7 @@
       </c>
       <c r="B404" t="inlineStr">
         <is>
-          <t>Muhammad</t>
+          <t>Koreshi</t>
         </is>
       </c>
       <c r="C404" t="n">
@@ -11811,7 +11811,7 @@
       </c>
       <c r="B409" t="inlineStr">
         <is>
-          <t>Mohy Ud Din</t>
+          <t>Zia</t>
         </is>
       </c>
       <c r="C409" t="n">
@@ -11832,7 +11832,7 @@
       </c>
       <c r="B410" t="inlineStr">
         <is>
-          <t>Zia</t>
+          <t>Hafiz Zia Ur Rehman</t>
         </is>
       </c>
       <c r="C410" t="n">
@@ -11853,7 +11853,7 @@
       </c>
       <c r="B411" t="inlineStr">
         <is>
-          <t>Hafiz Zia Ur Rehman</t>
+          <t>Mohy Ud Din</t>
         </is>
       </c>
       <c r="C411" t="n">
@@ -11958,7 +11958,7 @@
       </c>
       <c r="B416" t="inlineStr">
         <is>
-          <t>Mi Abbasi</t>
+          <t>Mh Dahri</t>
         </is>
       </c>
       <c r="C416" t="n">
@@ -11979,7 +11979,7 @@
       </c>
       <c r="B417" t="inlineStr">
         <is>
-          <t>Mh Dahri</t>
+          <t>Mi Abbasi</t>
         </is>
       </c>
       <c r="C417" t="n">
@@ -12021,7 +12021,7 @@
       </c>
       <c r="B419" t="inlineStr">
         <is>
-          <t>Muhammad Hashim Dahri</t>
+          <t>Muhammad Ramlee Kamarudin</t>
         </is>
       </c>
       <c r="C419" t="n">
@@ -12063,7 +12063,7 @@
       </c>
       <c r="B421" t="inlineStr">
         <is>
-          <t>Muhammad Ramlee Kamarudin</t>
+          <t>Yoshihide Yamada</t>
         </is>
       </c>
       <c r="C421" t="n">
@@ -12084,7 +12084,7 @@
       </c>
       <c r="B422" t="inlineStr">
         <is>
-          <t>Yoshihide Yamada</t>
+          <t>Muhammad Hashim Dahri</t>
         </is>
       </c>
       <c r="C422" t="n">
@@ -12126,7 +12126,7 @@
       </c>
       <c r="B424" t="inlineStr">
         <is>
-          <t>Subramaniam Ramesh</t>
+          <t>Sivathanu Chitra</t>
         </is>
       </c>
       <c r="C424" t="n">
@@ -12147,7 +12147,7 @@
       </c>
       <c r="B425" t="inlineStr">
         <is>
-          <t>Charles Vinoth</t>
+          <t>Joseph Charles Vinoth</t>
         </is>
       </c>
       <c r="C425" t="n">
@@ -12168,7 +12168,7 @@
       </c>
       <c r="B426" t="inlineStr">
         <is>
-          <t>Zuhairiah Z Abidin</t>
+          <t>Charles Vinoth</t>
         </is>
       </c>
       <c r="C426" t="n">
@@ -12189,7 +12189,7 @@
       </c>
       <c r="B427" t="inlineStr">
         <is>
-          <t>Elumalai Saranya</t>
+          <t>Zuhairiah Z Abidin</t>
         </is>
       </c>
       <c r="C427" t="n">
@@ -12210,7 +12210,7 @@
       </c>
       <c r="B428" t="inlineStr">
         <is>
-          <t>Sivathanu Chitra</t>
+          <t>Elumalai Saranya</t>
         </is>
       </c>
       <c r="C428" t="n">
@@ -12231,7 +12231,7 @@
       </c>
       <c r="B429" t="inlineStr">
         <is>
-          <t>Joseph Charles Vinoth</t>
+          <t>Subramaniam Ramesh</t>
         </is>
       </c>
       <c r="C429" t="n">
@@ -12357,7 +12357,7 @@
       </c>
       <c r="B435" t="inlineStr">
         <is>
-          <t>Mihai Datcu</t>
+          <t>Andrei Anghel</t>
         </is>
       </c>
       <c r="C435" t="n">
@@ -12378,7 +12378,7 @@
       </c>
       <c r="B436" t="inlineStr">
         <is>
-          <t>Andrei Anghel</t>
+          <t>Mihai Datcu</t>
         </is>
       </c>
       <c r="C436" t="n">
@@ -12441,7 +12441,7 @@
       </c>
       <c r="B439" t="inlineStr">
         <is>
-          <t>M Tzouvaras</t>
+          <t>E Kalogirou</t>
         </is>
       </c>
       <c r="C439" t="n">
@@ -12462,7 +12462,7 @@
       </c>
       <c r="B440" t="inlineStr">
         <is>
-          <t>E Kalogirou</t>
+          <t>D G Hadjimitsis</t>
         </is>
       </c>
       <c r="C440" t="n">
@@ -12483,7 +12483,7 @@
       </c>
       <c r="B441" t="inlineStr">
         <is>
-          <t>D G Hadjimitsis</t>
+          <t>D Makri</t>
         </is>
       </c>
       <c r="C441" t="n">
@@ -12504,7 +12504,7 @@
       </c>
       <c r="B442" t="inlineStr">
         <is>
-          <t>D Makri</t>
+          <t>C Mettas</t>
         </is>
       </c>
       <c r="C442" t="n">
@@ -12525,7 +12525,7 @@
       </c>
       <c r="B443" t="inlineStr">
         <is>
-          <t>C Mettas</t>
+          <t>M Tzouvaras</t>
         </is>
       </c>
       <c r="C443" t="n">
@@ -12609,7 +12609,7 @@
       </c>
       <c r="B447" t="inlineStr">
         <is>
-          <t>Samiullah Yousaf</t>
+          <t>Andrea Buono</t>
         </is>
       </c>
       <c r="C447" t="n">
@@ -12630,7 +12630,7 @@
       </c>
       <c r="B448" t="inlineStr">
         <is>
-          <t>Ferdinando Nunziata</t>
+          <t>Maurizio Migliaccio</t>
         </is>
       </c>
       <c r="C448" t="n">
@@ -12651,7 +12651,7 @@
       </c>
       <c r="B449" t="inlineStr">
         <is>
-          <t>Andrea Buono</t>
+          <t>Samiullah Yousaf</t>
         </is>
       </c>
       <c r="C449" t="n">
@@ -12672,7 +12672,7 @@
       </c>
       <c r="B450" t="inlineStr">
         <is>
-          <t>Maurizio Migliaccio</t>
+          <t>Ferdinando Nunziata</t>
         </is>
       </c>
       <c r="C450" t="n">
@@ -12714,7 +12714,7 @@
       </c>
       <c r="B452" t="inlineStr">
         <is>
-          <t>Omid Ghozatlou</t>
+          <t>Reza Mohammadi</t>
         </is>
       </c>
       <c r="C452" t="n">
@@ -12735,7 +12735,7 @@
       </c>
       <c r="B453" t="inlineStr">
         <is>
-          <t>Reza Mohammadi</t>
+          <t>Omid Ghozatlou</t>
         </is>
       </c>
       <c r="C453" t="n">
@@ -12987,7 +12987,7 @@
       </c>
       <c r="B465" t="inlineStr">
         <is>
-          <t>R Tong</t>
+          <t>M Shakeel</t>
         </is>
       </c>
       <c r="C465" t="n">
@@ -13008,7 +13008,7 @@
       </c>
       <c r="B466" t="inlineStr">
         <is>
-          <t>M Shakeel</t>
+          <t>R Tong</t>
         </is>
       </c>
       <c r="C466" t="n">
@@ -13050,7 +13050,7 @@
       </c>
       <c r="B468" t="inlineStr">
         <is>
-          <t>Rizwan Ullah</t>
+          <t>Md Shohidul Islam</t>
         </is>
       </c>
       <c r="C468" t="n">
@@ -13071,7 +13071,7 @@
       </c>
       <c r="B469" t="inlineStr">
         <is>
-          <t>Md Shohidul Islam</t>
+          <t>Rizwan Ullah</t>
         </is>
       </c>
       <c r="C469" t="n">
@@ -13155,7 +13155,7 @@
       </c>
       <c r="B473" t="inlineStr">
         <is>
-          <t>Imtiaz</t>
+          <t>Rabia Afrasiab</t>
         </is>
       </c>
       <c r="C473" t="n">
@@ -13176,7 +13176,7 @@
       </c>
       <c r="B474" t="inlineStr">
         <is>
-          <t>Asma Talib Qureshi</t>
+          <t>Imtiaz</t>
         </is>
       </c>
       <c r="C474" t="n">
@@ -13197,7 +13197,7 @@
       </c>
       <c r="B475" t="inlineStr">
         <is>
-          <t>Rabia Afrasiab</t>
+          <t>Asma Talib Qureshi</t>
         </is>
       </c>
       <c r="C475" t="n">
@@ -13302,7 +13302,7 @@
       </c>
       <c r="B480" t="inlineStr">
         <is>
-          <t>Waqas Ahmed</t>
+          <t>Rizwan Ahmed</t>
         </is>
       </c>
       <c r="C480" t="n">
@@ -13323,7 +13323,7 @@
       </c>
       <c r="B481" t="inlineStr">
         <is>
-          <t>Rizwan Ahmed</t>
+          <t>Waqas Ahmed</t>
         </is>
       </c>
       <c r="C481" t="n">
@@ -13344,7 +13344,7 @@
       </c>
       <c r="B482" t="inlineStr">
         <is>
-          <t>Emilie Avignon</t>
+          <t>Philippe Bénabès</t>
         </is>
       </c>
       <c r="C482" t="n">
@@ -13365,7 +13365,7 @@
       </c>
       <c r="B483" t="inlineStr">
         <is>
-          <t>Mohamed Ben Chouikha</t>
+          <t>Caroline Lelandais Perrault</t>
         </is>
       </c>
       <c r="C483" t="n">
@@ -13386,7 +13386,7 @@
       </c>
       <c r="B484" t="inlineStr">
         <is>
-          <t>Philippe Bénabès</t>
+          <t>Mohamed Ben Chouikha</t>
         </is>
       </c>
       <c r="C484" t="n">
@@ -13428,7 +13428,7 @@
       </c>
       <c r="B486" t="inlineStr">
         <is>
-          <t>Caroline Lelandais Perrault</t>
+          <t>Emilie Avignon</t>
         </is>
       </c>
       <c r="C486" t="n">
@@ -13491,7 +13491,7 @@
       </c>
       <c r="B489" t="inlineStr">
         <is>
-          <t>Nabil El Ioini</t>
+          <t>Hamid R Barzegar</t>
         </is>
       </c>
       <c r="C489" t="n">
@@ -13512,7 +13512,7 @@
       </c>
       <c r="B490" t="inlineStr">
         <is>
-          <t>Hamid R Barzegar</t>
+          <t>Nabil El Ioini</t>
         </is>
       </c>
       <c r="C490" t="n">
@@ -13575,7 +13575,7 @@
       </c>
       <c r="B493" t="inlineStr">
         <is>
-          <t>Abdul Wahab</t>
+          <t>Kashif Hussain</t>
         </is>
       </c>
       <c r="C493" t="n">
@@ -13596,7 +13596,7 @@
       </c>
       <c r="B494" t="inlineStr">
         <is>
-          <t>Tahir Bashir</t>
+          <t>Abdul Wahab</t>
         </is>
       </c>
       <c r="C494" t="n">
@@ -13638,7 +13638,7 @@
       </c>
       <c r="B496" t="inlineStr">
         <is>
-          <t>Haroon Ahmed</t>
+          <t>Tahir Bashir</t>
         </is>
       </c>
       <c r="C496" t="n">
@@ -13659,7 +13659,7 @@
       </c>
       <c r="B497" t="inlineStr">
         <is>
-          <t>Kashif Hussain</t>
+          <t>Haroon Ahmed</t>
         </is>
       </c>
       <c r="C497" t="n">
@@ -13722,7 +13722,7 @@
       </c>
       <c r="B500" t="inlineStr">
         <is>
-          <t>Yiqi Cheng</t>
+          <t>Xinhua Wang</t>
         </is>
       </c>
       <c r="C500" t="n">
@@ -13743,7 +13743,7 @@
       </c>
       <c r="B501" t="inlineStr">
         <is>
-          <t>Xinhua Wang</t>
+          <t>Yiqi Cheng</t>
         </is>
       </c>
       <c r="C501" t="n">
@@ -13806,7 +13806,7 @@
       </c>
       <c r="B504" t="inlineStr">
         <is>
-          <t>Yongming Li</t>
+          <t>Zhiyong Huang</t>
         </is>
       </c>
       <c r="C504" t="n">
@@ -13827,7 +13827,7 @@
       </c>
       <c r="B505" t="inlineStr">
         <is>
-          <t>Mingyao Yang</t>
+          <t>Yongming Li</t>
         </is>
       </c>
       <c r="C505" t="n">
@@ -13869,7 +13869,7 @@
       </c>
       <c r="B507" t="inlineStr">
         <is>
-          <t>Zhiyong Huang</t>
+          <t>Jie Ma</t>
         </is>
       </c>
       <c r="C507" t="n">
@@ -13890,7 +13890,7 @@
       </c>
       <c r="B508" t="inlineStr">
         <is>
-          <t>Jie Ma</t>
+          <t>Mingyao Yang</t>
         </is>
       </c>
       <c r="C508" t="n">
@@ -13911,7 +13911,7 @@
       </c>
       <c r="B509" t="inlineStr">
         <is>
-          <t>Nasim Ullah</t>
+          <t>Fahad R Albogamy</t>
         </is>
       </c>
       <c r="C509" t="n">
@@ -13953,7 +13953,7 @@
       </c>
       <c r="B511" t="inlineStr">
         <is>
-          <t>Fahad R Albogamy</t>
+          <t>Nasim Ullah</t>
         </is>
       </c>
       <c r="C511" t="n">
@@ -14016,7 +14016,7 @@
       </c>
       <c r="B514" t="inlineStr">
         <is>
-          <t>Jun Bae Seo</t>
+          <t>Hu Jin</t>
         </is>
       </c>
       <c r="C514" t="n">
@@ -14037,7 +14037,7 @@
       </c>
       <c r="B515" t="inlineStr">
         <is>
-          <t>Hu Jin</t>
+          <t>Jun Bae Seo</t>
         </is>
       </c>
       <c r="C515" t="n">
@@ -14079,7 +14079,7 @@
       </c>
       <c r="B517" t="inlineStr">
         <is>
-          <t>Naeem Maroof</t>
+          <t>Saqib Ali Khan</t>
         </is>
       </c>
       <c r="C517" t="n">
@@ -14100,7 +14100,7 @@
       </c>
       <c r="B518" t="inlineStr">
         <is>
-          <t>Saqib Ali Khan</t>
+          <t>Naeem Maroof</t>
         </is>
       </c>
       <c r="C518" t="n">
@@ -14310,7 +14310,7 @@
       </c>
       <c r="B528" t="inlineStr">
         <is>
-          <t>Atiqa Saeed</t>
+          <t>Muhammad Umair Ahmad Khan</t>
         </is>
       </c>
       <c r="C528" t="n">
@@ -14352,7 +14352,7 @@
       </c>
       <c r="B530" t="inlineStr">
         <is>
-          <t>Muhammad Umair Ahmad Khan</t>
+          <t>Atiqa Saeed</t>
         </is>
       </c>
       <c r="C530" t="n">
@@ -14373,7 +14373,7 @@
       </c>
       <c r="B531" t="inlineStr">
         <is>
-          <t>Faiza Bibi</t>
+          <t>Zaryab Basharat</t>
         </is>
       </c>
       <c r="C531" t="n">
@@ -14394,7 +14394,7 @@
       </c>
       <c r="B532" t="inlineStr">
         <is>
-          <t>Zaryab Basharat</t>
+          <t>Saqlain Abbas</t>
         </is>
       </c>
       <c r="C532" t="n">
@@ -14415,7 +14415,7 @@
       </c>
       <c r="B533" t="inlineStr">
         <is>
-          <t>Zulkarnain Abbas</t>
+          <t>Ahmad Ali</t>
         </is>
       </c>
       <c r="C533" t="n">
@@ -14436,7 +14436,7 @@
       </c>
       <c r="B534" t="inlineStr">
         <is>
-          <t>Ahmad Ali</t>
+          <t>Komal Afzal</t>
         </is>
       </c>
       <c r="C534" t="n">
@@ -14478,7 +14478,7 @@
       </c>
       <c r="B536" t="inlineStr">
         <is>
-          <t>Saqlain Abbas</t>
+          <t>Zulkarnain Abbas</t>
         </is>
       </c>
       <c r="C536" t="n">
@@ -14499,7 +14499,7 @@
       </c>
       <c r="B537" t="inlineStr">
         <is>
-          <t>Komal Afzal</t>
+          <t>Faiza Bibi</t>
         </is>
       </c>
       <c r="C537" t="n">
@@ -14520,7 +14520,7 @@
       </c>
       <c r="B538" t="inlineStr">
         <is>
-          <t>Sherazi</t>
+          <t>Nimra Saleem</t>
         </is>
       </c>
       <c r="C538" t="n">
@@ -14541,7 +14541,7 @@
       </c>
       <c r="B539" t="inlineStr">
         <is>
-          <t>Abdullah Khan</t>
+          <t>Sherazi</t>
         </is>
       </c>
       <c r="C539" t="n">
@@ -14562,7 +14562,7 @@
       </c>
       <c r="B540" t="inlineStr">
         <is>
-          <t>Nimra Saleem</t>
+          <t>Abdullah Khan</t>
         </is>
       </c>
       <c r="C540" t="n">
@@ -14604,7 +14604,7 @@
       </c>
       <c r="B542" t="inlineStr">
         <is>
-          <t>Muhammad Masab</t>
+          <t>Mujeeb Ur Rehman</t>
         </is>
       </c>
       <c r="C542" t="n">
@@ -14625,7 +14625,7 @@
       </c>
       <c r="B543" t="inlineStr">
         <is>
-          <t>Mujeeb Ur Rehman</t>
+          <t>Muhammad Masab</t>
         </is>
       </c>
       <c r="C543" t="n">
@@ -14646,7 +14646,7 @@
       </c>
       <c r="B544" t="inlineStr">
         <is>
-          <t>Farhat Masood</t>
+          <t>Rabeel Manzoor</t>
         </is>
       </c>
       <c r="C544" t="n">
@@ -14667,7 +14667,7 @@
       </c>
       <c r="B545" t="inlineStr">
         <is>
-          <t>Rabeel Manzoor</t>
+          <t>Sanika K Wijayasekara</t>
         </is>
       </c>
       <c r="C545" t="n">
@@ -14688,7 +14688,7 @@
       </c>
       <c r="B546" t="inlineStr">
         <is>
-          <t>Sanika K Wijayasekara</t>
+          <t>Farhat Masood</t>
         </is>
       </c>
       <c r="C546" t="n">
@@ -14772,7 +14772,7 @@
       </c>
       <c r="B550" t="inlineStr">
         <is>
-          <t>Muhammad Talha Noor</t>
+          <t>Shahid Mumtaz</t>
         </is>
       </c>
       <c r="C550" t="n">
@@ -14793,7 +14793,7 @@
       </c>
       <c r="B551" t="inlineStr">
         <is>
-          <t>Shahid Mumtaz</t>
+          <t>Muhammad Talha Noor</t>
         </is>
       </c>
       <c r="C551" t="n">
@@ -14856,7 +14856,7 @@
       </c>
       <c r="B554" t="inlineStr">
         <is>
-          <t>Hafsa Amanullah</t>
+          <t>Dost Muhammad</t>
         </is>
       </c>
       <c r="C554" t="n">
@@ -14877,7 +14877,7 @@
       </c>
       <c r="B555" t="inlineStr">
         <is>
-          <t>Dost Muhammad</t>
+          <t>Manuel Mazzara</t>
         </is>
       </c>
       <c r="C555" t="n">
@@ -14898,7 +14898,7 @@
       </c>
       <c r="B556" t="inlineStr">
         <is>
-          <t>Manuel Mazzara</t>
+          <t>Hafsa Amanullah</t>
         </is>
       </c>
       <c r="C556" t="n">
@@ -14919,7 +14919,7 @@
       </c>
       <c r="B557" t="inlineStr">
         <is>
-          <t>Muhammad Ahmad</t>
+          <t>Saqib Bhatti</t>
         </is>
       </c>
       <c r="C557" t="n">
@@ -14940,7 +14940,7 @@
       </c>
       <c r="B558" t="inlineStr">
         <is>
-          <t>Saqib Bhatti</t>
+          <t>Muhammad Ahmad</t>
         </is>
       </c>
       <c r="C558" t="n">
@@ -14982,7 +14982,7 @@
       </c>
       <c r="B560" t="inlineStr">
         <is>
-          <t>Ogobuchi Daniel Okey</t>
+          <t>Dick Carrillo Melgarejo</t>
         </is>
       </c>
       <c r="C560" t="n">
@@ -15003,7 +15003,7 @@
       </c>
       <c r="B561" t="inlineStr">
         <is>
-          <t>Dick Carrillo Melgarejo</t>
+          <t>Siti Sarah Maidin</t>
         </is>
       </c>
       <c r="C561" t="n">
@@ -15024,7 +15024,7 @@
       </c>
       <c r="B562" t="inlineStr">
         <is>
-          <t>Siti Sarah Maidin</t>
+          <t>Renata Lopes Rosa</t>
         </is>
       </c>
       <c r="C562" t="n">
@@ -15045,7 +15045,7 @@
       </c>
       <c r="B563" t="inlineStr">
         <is>
-          <t>Renata Lopes Rosa</t>
+          <t>Ogobuchi Daniel Okey</t>
         </is>
       </c>
       <c r="C563" t="n">
@@ -15066,7 +15066,7 @@
       </c>
       <c r="B564" t="inlineStr">
         <is>
-          <t>Zafar Baig</t>
+          <t>Asif Hussain</t>
         </is>
       </c>
       <c r="C564" t="n">
@@ -15087,7 +15087,7 @@
       </c>
       <c r="B565" t="inlineStr">
         <is>
-          <t>Tamara Al Shloul</t>
+          <t>Zafar Baig</t>
         </is>
       </c>
       <c r="C565" t="n">
@@ -15108,7 +15108,7 @@
       </c>
       <c r="B566" t="inlineStr">
         <is>
-          <t>Asif Hussain</t>
+          <t>Tamara Al Shloul</t>
         </is>
       </c>
       <c r="C566" t="n">
@@ -15150,7 +15150,7 @@
       </c>
       <c r="B568" t="inlineStr">
         <is>
-          <t>Mohamed R Abonazel</t>
+          <t>Muhammad Adnan</t>
         </is>
       </c>
       <c r="C568" t="n">
@@ -15171,7 +15171,7 @@
       </c>
       <c r="B569" t="inlineStr">
         <is>
-          <t>Muhammad Asim Butt</t>
+          <t>Syed Rehan Ashraf</t>
         </is>
       </c>
       <c r="C569" t="n">
@@ -15213,7 +15213,7 @@
       </c>
       <c r="B571" t="inlineStr">
         <is>
-          <t>Muhammad Adnan</t>
+          <t>Izaz Hassan</t>
         </is>
       </c>
       <c r="C571" t="n">
@@ -15234,7 +15234,7 @@
       </c>
       <c r="B572" t="inlineStr">
         <is>
-          <t>Izaz Hassan</t>
+          <t>Fuad A Awwad</t>
         </is>
       </c>
       <c r="C572" t="n">
@@ -15255,7 +15255,7 @@
       </c>
       <c r="B573" t="inlineStr">
         <is>
-          <t>Syed Rehan Ashraf</t>
+          <t>Khalid Ijaz</t>
         </is>
       </c>
       <c r="C573" t="n">
@@ -15276,7 +15276,7 @@
       </c>
       <c r="B574" t="inlineStr">
         <is>
-          <t>Fuad A Awwad</t>
+          <t>Mohamed R Abonazel</t>
         </is>
       </c>
       <c r="C574" t="n">
@@ -15297,7 +15297,7 @@
       </c>
       <c r="B575" t="inlineStr">
         <is>
-          <t>Khalid Ijaz</t>
+          <t>Muhammad Asim Butt</t>
         </is>
       </c>
       <c r="C575" t="n">
@@ -15339,7 +15339,7 @@
       </c>
       <c r="B577" t="inlineStr">
         <is>
-          <t>Amira Syed A Aziz</t>
+          <t>El Awadi Attia</t>
         </is>
       </c>
       <c r="C577" t="n">
@@ -15360,7 +15360,7 @@
       </c>
       <c r="B578" t="inlineStr">
         <is>
-          <t>El Awadi Attia</t>
+          <t>Amira Syed A Aziz</t>
         </is>
       </c>
       <c r="C578" t="n">
@@ -15423,7 +15423,7 @@
       </c>
       <c r="B581" t="inlineStr">
         <is>
-          <t>Muhammad Shoaib</t>
+          <t>Saddique Khalid</t>
         </is>
       </c>
       <c r="C581" t="n">
@@ -15465,7 +15465,7 @@
       </c>
       <c r="B583" t="inlineStr">
         <is>
-          <t>Saddique Khalid</t>
+          <t>Muhammad Shoaib</t>
         </is>
       </c>
       <c r="C583" t="n">
@@ -15486,7 +15486,7 @@
       </c>
       <c r="B584" t="inlineStr">
         <is>
-          <t>Toseeq Haider Bajwa</t>
+          <t>Umair Bajwa</t>
         </is>
       </c>
       <c r="C584" t="n">
@@ -15507,7 +15507,7 @@
       </c>
       <c r="B585" t="inlineStr">
         <is>
-          <t>Umair Bajwa</t>
+          <t>Toseeq Haider Bajwa</t>
         </is>
       </c>
       <c r="C585" t="n">
@@ -15633,7 +15633,7 @@
       </c>
       <c r="B591" t="inlineStr">
         <is>
-          <t>Maania Jabbar</t>
+          <t>Farah Khalid</t>
         </is>
       </c>
       <c r="C591" t="n">
@@ -15654,7 +15654,7 @@
       </c>
       <c r="B592" t="inlineStr">
         <is>
-          <t>Farah Khalid</t>
+          <t>Muhammad Farhan</t>
         </is>
       </c>
       <c r="C592" t="n">
@@ -15696,7 +15696,7 @@
       </c>
       <c r="B594" t="inlineStr">
         <is>
-          <t>Muhammad Farhan</t>
+          <t>Maania Jabbar</t>
         </is>
       </c>
       <c r="C594" t="n">
@@ -15906,7 +15906,7 @@
       </c>
       <c r="B604" t="inlineStr">
         <is>
-          <t>A M Jaradat</t>
+          <t>M I Sağlam</t>
         </is>
       </c>
       <c r="C604" t="n">
@@ -15927,7 +15927,7 @@
       </c>
       <c r="B605" t="inlineStr">
         <is>
-          <t>M I Sağlam</t>
+          <t>M Kartal</t>
         </is>
       </c>
       <c r="C605" t="n">
@@ -15948,7 +15948,7 @@
       </c>
       <c r="B606" t="inlineStr">
         <is>
-          <t>M Kartal</t>
+          <t>A M Jaradat</t>
         </is>
       </c>
       <c r="C606" t="n">
@@ -16011,7 +16011,7 @@
       </c>
       <c r="B609" t="inlineStr">
         <is>
-          <t>Mamady Delamou</t>
+          <t>El Mehdi Amhoud</t>
         </is>
       </c>
       <c r="C609" t="n">
@@ -16032,7 +16032,7 @@
       </c>
       <c r="B610" t="inlineStr">
         <is>
-          <t>El Mehdi Amhoud</t>
+          <t>Mamady Delamou</t>
         </is>
       </c>
       <c r="C610" t="n">
@@ -16116,7 +16116,7 @@
       </c>
       <c r="B614" t="inlineStr">
         <is>
-          <t>Adnan Zafar</t>
+          <t>Ashfaq Ahmed</t>
         </is>
       </c>
       <c r="C614" t="n">
@@ -16137,7 +16137,7 @@
       </c>
       <c r="B615" t="inlineStr">
         <is>
-          <t>Ashfaq Ahmed</t>
+          <t>Adnan Zafar</t>
         </is>
       </c>
       <c r="C615" t="n">
@@ -16158,7 +16158,7 @@
       </c>
       <c r="B616" t="inlineStr">
         <is>
-          <t>Hassaan Khaliq</t>
+          <t>Qureshi</t>
         </is>
       </c>
       <c r="C616" t="n">
@@ -16179,7 +16179,7 @@
       </c>
       <c r="B617" t="inlineStr">
         <is>
-          <t>Qureshi</t>
+          <t>Hassaan Khaliq</t>
         </is>
       </c>
       <c r="C617" t="n">
@@ -16326,7 +16326,7 @@
       </c>
       <c r="B624" t="inlineStr">
         <is>
-          <t>Qiang Lu</t>
+          <t>Chang Qing Dong</t>
         </is>
       </c>
       <c r="C624" t="n">
@@ -16347,7 +16347,7 @@
       </c>
       <c r="B625" t="inlineStr">
         <is>
-          <t>Adnan Abbas</t>
+          <t>Qiang Lu</t>
         </is>
       </c>
       <c r="C625" t="n">
@@ -16368,7 +16368,7 @@
       </c>
       <c r="B626" t="inlineStr">
         <is>
-          <t>Chang Qing Dong</t>
+          <t>Zulfiqar Ali</t>
         </is>
       </c>
       <c r="C626" t="n">
@@ -16389,7 +16389,7 @@
       </c>
       <c r="B627" t="inlineStr">
         <is>
-          <t>Zulfiqar Ali</t>
+          <t>Zafar Hussain</t>
         </is>
       </c>
       <c r="C627" t="n">
@@ -16410,7 +16410,7 @@
       </c>
       <c r="B628" t="inlineStr">
         <is>
-          <t>Zafar Hussain</t>
+          <t>Adnan Abbas</t>
         </is>
       </c>
       <c r="C628" t="n">
@@ -16473,7 +16473,7 @@
       </c>
       <c r="B631" t="inlineStr">
         <is>
-          <t>Zahid Ali</t>
+          <t>Danyal Asif</t>
         </is>
       </c>
       <c r="C631" t="n">
@@ -16494,7 +16494,7 @@
       </c>
       <c r="B632" t="inlineStr">
         <is>
-          <t>Danyal Asif</t>
+          <t>Zahid Ali</t>
         </is>
       </c>
       <c r="C632" t="n">
@@ -16515,7 +16515,7 @@
       </c>
       <c r="B633" t="inlineStr">
         <is>
-          <t>Li Meicheng</t>
+          <t>Mohan Menghwar</t>
         </is>
       </c>
       <c r="C633" t="n">
@@ -16536,7 +16536,7 @@
       </c>
       <c r="B634" t="inlineStr">
         <is>
-          <t>Mohan Menghwar</t>
+          <t>Li Meicheng</t>
         </is>
       </c>
       <c r="C634" t="n">
@@ -16620,7 +16620,7 @@
       </c>
       <c r="B638" t="inlineStr">
         <is>
-          <t>Kai Yi</t>
+          <t>Chengrong Li</t>
         </is>
       </c>
       <c r="C638" t="n">
@@ -16641,7 +16641,7 @@
       </c>
       <c r="B639" t="inlineStr">
         <is>
-          <t>Chengrong Li</t>
+          <t>Yuzhen Lv</t>
         </is>
       </c>
       <c r="C639" t="n">
@@ -16683,7 +16683,7 @@
       </c>
       <c r="B641" t="inlineStr">
         <is>
-          <t>Yuzhen Lv</t>
+          <t>Kai Yi</t>
         </is>
       </c>
       <c r="C641" t="n">
@@ -16704,7 +16704,7 @@
       </c>
       <c r="B642" t="inlineStr">
         <is>
-          <t>Syed Furqan Rafique</t>
+          <t>Farukh Abbas</t>
         </is>
       </c>
       <c r="C642" t="n">
@@ -16725,7 +16725,7 @@
       </c>
       <c r="B643" t="inlineStr">
         <is>
-          <t>Farukh Abbas</t>
+          <t>Syed Furqan Rafique</t>
         </is>
       </c>
       <c r="C643" t="n">
@@ -16830,7 +16830,7 @@
       </c>
       <c r="B648" t="inlineStr">
         <is>
-          <t>Saad A Butt</t>
+          <t>Hassan A Khan</t>
         </is>
       </c>
       <c r="C648" t="n">
@@ -16851,7 +16851,7 @@
       </c>
       <c r="B649" t="inlineStr">
         <is>
-          <t>Hassan A Khan</t>
+          <t>Saad A Butt</t>
         </is>
       </c>
       <c r="C649" t="n">
@@ -16893,7 +16893,7 @@
       </c>
       <c r="B651" t="inlineStr">
         <is>
-          <t>Hassan Abbas Khan</t>
+          <t>Syed Muhammad Ahsan</t>
         </is>
       </c>
       <c r="C651" t="n">
@@ -16914,7 +16914,7 @@
       </c>
       <c r="B652" t="inlineStr">
         <is>
-          <t>Syed Muhammad Ahsan</t>
+          <t>Nauman Ahmad Zaffar</t>
         </is>
       </c>
       <c r="C652" t="n">
@@ -16935,7 +16935,7 @@
       </c>
       <c r="B653" t="inlineStr">
         <is>
-          <t>Nauman Ahmad Zaffar</t>
+          <t>Hassan Abbas Khan</t>
         </is>
       </c>
       <c r="C653" t="n">
@@ -17019,7 +17019,7 @@
       </c>
       <c r="B657" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>K</t>
         </is>
       </c>
       <c r="C657" t="n">
@@ -17040,7 +17040,7 @@
       </c>
       <c r="B658" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>Fujii</t>
         </is>
       </c>
       <c r="C658" t="n">
@@ -17061,7 +17061,7 @@
       </c>
       <c r="B659" t="inlineStr">
         <is>
-          <t>Fujii</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="C659" t="n">
@@ -17166,7 +17166,7 @@
       </c>
       <c r="B664" t="inlineStr">
         <is>
-          <t>M R</t>
+          <t>R Abdul Karim</t>
         </is>
       </c>
       <c r="C664" t="n">
@@ -17187,7 +17187,7 @@
       </c>
       <c r="B665" t="inlineStr">
         <is>
-          <t>R Abdul Karim</t>
+          <t>M R</t>
         </is>
       </c>
       <c r="C665" t="n">
@@ -17229,7 +17229,7 @@
       </c>
       <c r="B667" t="inlineStr">
         <is>
-          <t>Marwat</t>
+          <t>M R A</t>
         </is>
       </c>
       <c r="C667" t="n">
@@ -17250,7 +17250,7 @@
       </c>
       <c r="B668" t="inlineStr">
         <is>
-          <t>M R A</t>
+          <t>Marwat</t>
         </is>
       </c>
       <c r="C668" t="n">
@@ -17313,7 +17313,7 @@
       </c>
       <c r="B671" t="inlineStr">
         <is>
-          <t>Daas</t>
+          <t>T H</t>
         </is>
       </c>
       <c r="C671" t="n">
@@ -17334,7 +17334,7 @@
       </c>
       <c r="B672" t="inlineStr">
         <is>
-          <t>M M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="C672" t="n">
@@ -17376,7 +17376,7 @@
       </c>
       <c r="B674" t="inlineStr">
         <is>
-          <t>Haider</t>
+          <t>M M</t>
         </is>
       </c>
       <c r="C674" t="n">
@@ -17397,7 +17397,7 @@
       </c>
       <c r="B675" t="inlineStr">
         <is>
-          <t>T H</t>
+          <t>Haider</t>
         </is>
       </c>
       <c r="C675" t="n">
@@ -17418,7 +17418,7 @@
       </c>
       <c r="B676" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>Daas</t>
         </is>
       </c>
       <c r="C676" t="n">
@@ -17481,7 +17481,7 @@
       </c>
       <c r="B679" t="inlineStr">
         <is>
-          <t>Kurochkin</t>
+          <t>A A</t>
         </is>
       </c>
       <c r="C679" t="n">
@@ -17502,7 +17502,7 @@
       </c>
       <c r="B680" t="inlineStr">
         <is>
-          <t>A A</t>
+          <t>Y S</t>
         </is>
       </c>
       <c r="C680" t="n">
@@ -17523,7 +17523,7 @@
       </c>
       <c r="B681" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C681" t="n">
@@ -17544,7 +17544,7 @@
       </c>
       <c r="B682" t="inlineStr">
         <is>
-          <t>Y S</t>
+          <t>Razumtecev</t>
         </is>
       </c>
       <c r="C682" t="n">
@@ -17565,7 +17565,7 @@
       </c>
       <c r="B683" t="inlineStr">
         <is>
-          <t>Kolesnikov</t>
+          <t>I</t>
         </is>
       </c>
       <c r="C683" t="n">
@@ -17586,7 +17586,7 @@
       </c>
       <c r="B684" t="inlineStr">
         <is>
-          <t>Razumtecev</t>
+          <t>Kolesnikov</t>
         </is>
       </c>
       <c r="C684" t="n">
@@ -17607,7 +17607,7 @@
       </c>
       <c r="B685" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Kurochkin</t>
         </is>
       </c>
       <c r="C685" t="n">
@@ -17628,7 +17628,7 @@
       </c>
       <c r="B686" t="inlineStr">
         <is>
-          <t>Momna Ikram</t>
+          <t>Walaa Alayed</t>
         </is>
       </c>
       <c r="C686" t="n">
@@ -17649,7 +17649,7 @@
       </c>
       <c r="B687" t="inlineStr">
         <is>
-          <t>Walaa Alayed</t>
+          <t>Momna Ikram</t>
         </is>
       </c>
       <c r="C687" t="n">
@@ -17670,7 +17670,7 @@
       </c>
       <c r="B688" t="inlineStr">
         <is>
-          <t>Zaheer Asghar</t>
+          <t>Ahmed Zeeshan</t>
         </is>
       </c>
       <c r="C688" t="n">
@@ -17691,7 +17691,7 @@
       </c>
       <c r="B689" t="inlineStr">
         <is>
-          <t>Dilawar Hussain</t>
+          <t>Zaheer Asghar</t>
         </is>
       </c>
       <c r="C689" t="n">
@@ -17712,7 +17712,7 @@
       </c>
       <c r="B690" t="inlineStr">
         <is>
-          <t>Ahmed Zeeshan</t>
+          <t>Dilawar Hussain</t>
         </is>
       </c>
       <c r="C690" t="n">
@@ -17733,7 +17733,7 @@
       </c>
       <c r="B691" t="inlineStr">
         <is>
-          <t>Anas Alsuhaibani</t>
+          <t>Youssef N Altherwy</t>
         </is>
       </c>
       <c r="C691" t="n">
@@ -17754,7 +17754,7 @@
       </c>
       <c r="B692" t="inlineStr">
         <is>
-          <t>Bilal Ahmed</t>
+          <t>Syed Rameez Naqvi</t>
         </is>
       </c>
       <c r="C692" t="n">
@@ -17775,7 +17775,7 @@
       </c>
       <c r="B693" t="inlineStr">
         <is>
-          <t>Tallha Akram</t>
+          <t>Bilal Ahmed</t>
         </is>
       </c>
       <c r="C693" t="n">
@@ -17796,7 +17796,7 @@
       </c>
       <c r="B694" t="inlineStr">
         <is>
-          <t>Youssef N Altherwy</t>
+          <t>Tallha Akram</t>
         </is>
       </c>
       <c r="C694" t="n">
@@ -17817,7 +17817,7 @@
       </c>
       <c r="B695" t="inlineStr">
         <is>
-          <t>Syed Rameez Naqvi</t>
+          <t>Anas Alsuhaibani</t>
         </is>
       </c>
       <c r="C695" t="n">
@@ -17838,7 +17838,7 @@
       </c>
       <c r="B696" t="inlineStr">
         <is>
-          <t>Gulistan Raja</t>
+          <t>Qaiser Hussain</t>
         </is>
       </c>
       <c r="C696" t="n">
@@ -17859,7 +17859,7 @@
       </c>
       <c r="B697" t="inlineStr">
         <is>
-          <t>Qaiser Hussain</t>
+          <t>Gulistan Raja</t>
         </is>
       </c>
       <c r="C697" t="n">
@@ -17964,7 +17964,7 @@
       </c>
       <c r="B702" t="inlineStr">
         <is>
-          <t>Aamir Mahmood</t>
+          <t>Mikael Gidlund</t>
         </is>
       </c>
       <c r="C702" t="n">
@@ -17985,7 +17985,7 @@
       </c>
       <c r="B703" t="inlineStr">
         <is>
-          <t>Mikael Gidlund</t>
+          <t>Aamir Mahmood</t>
         </is>
       </c>
       <c r="C703" t="n">
@@ -18216,7 +18216,7 @@
       </c>
       <c r="B714" t="inlineStr">
         <is>
-          <t>Amir Haider</t>
+          <t>Rashid Ali</t>
         </is>
       </c>
       <c r="C714" t="n">
@@ -18237,7 +18237,7 @@
       </c>
       <c r="B715" t="inlineStr">
         <is>
-          <t>Rashid Ali</t>
+          <t>Amir Haider</t>
         </is>
       </c>
       <c r="C715" t="n">
@@ -18405,7 +18405,7 @@
       </c>
       <c r="B723" t="inlineStr">
         <is>
-          <t>Sarim Farqaleet Khan</t>
+          <t>Umais Khan</t>
         </is>
       </c>
       <c r="C723" t="n">
@@ -18426,7 +18426,7 @@
       </c>
       <c r="B724" t="inlineStr">
         <is>
-          <t>Umais Khan</t>
+          <t>Sarim Farqaleet Khan</t>
         </is>
       </c>
       <c r="C724" t="n">
@@ -18468,7 +18468,7 @@
       </c>
       <c r="B726" t="inlineStr">
         <is>
-          <t>Abraiz Khattak</t>
+          <t>Iu Khalil</t>
         </is>
       </c>
       <c r="C726" t="n">
@@ -18489,7 +18489,7 @@
       </c>
       <c r="B727" t="inlineStr">
         <is>
-          <t>Iu Khalil</t>
+          <t>Abraiz Khattak</t>
         </is>
       </c>
       <c r="C727" t="n">
@@ -18552,7 +18552,7 @@
       </c>
       <c r="B730" t="inlineStr">
         <is>
-          <t>Wadood Abdul</t>
+          <t>Imtiaz Ahmed Taj</t>
         </is>
       </c>
       <c r="C730" t="n">
@@ -18573,7 +18573,7 @@
       </c>
       <c r="B731" t="inlineStr">
         <is>
-          <t>Imtiaz Ahmed Taj</t>
+          <t>Wadood Abdul</t>
         </is>
       </c>
       <c r="C731" t="n">
@@ -18678,7 +18678,7 @@
       </c>
       <c r="B736" t="inlineStr">
         <is>
-          <t>Saifullah Khan</t>
+          <t>Qudratullah Wazir</t>
         </is>
       </c>
       <c r="C736" t="n">
@@ -18699,7 +18699,7 @@
       </c>
       <c r="B737" t="inlineStr">
         <is>
-          <t>Faiza Hayat</t>
+          <t>Saifullah Khan</t>
         </is>
       </c>
       <c r="C737" t="n">
@@ -18720,7 +18720,7 @@
       </c>
       <c r="B738" t="inlineStr">
         <is>
-          <t>Qudratullah Wazir</t>
+          <t>Faiza Hayat</t>
         </is>
       </c>
       <c r="C738" t="n">
@@ -18972,7 +18972,7 @@
       </c>
       <c r="B750" t="inlineStr">
         <is>
-          <t>Atif Naveed Khan</t>
+          <t>Muhammad Nadeem</t>
         </is>
       </c>
       <c r="C750" t="n">
@@ -18993,7 +18993,7 @@
       </c>
       <c r="B751" t="inlineStr">
         <is>
-          <t>Muhammad Nadeem</t>
+          <t>Atif Naveed Khan</t>
         </is>
       </c>
       <c r="C751" t="n">
@@ -19014,7 +19014,7 @@
       </c>
       <c r="B752" t="inlineStr">
         <is>
-          <t>Masood Khan</t>
+          <t>Shahzad Younis</t>
         </is>
       </c>
       <c r="C752" t="n">
@@ -19056,7 +19056,7 @@
       </c>
       <c r="B754" t="inlineStr">
         <is>
-          <t>Shahzad Younis</t>
+          <t>Abdul Kashif Janjua</t>
         </is>
       </c>
       <c r="C754" t="n">
@@ -19077,7 +19077,7 @@
       </c>
       <c r="B755" t="inlineStr">
         <is>
-          <t>Abdul Kashif Janjua</t>
+          <t>Masood Khan</t>
         </is>
       </c>
       <c r="C755" t="n">
@@ -19329,7 +19329,7 @@
       </c>
       <c r="B767" t="inlineStr">
         <is>
-          <t>Bakhtiar Ul Haq</t>
+          <t>Abdul Shakoor</t>
         </is>
       </c>
       <c r="C767" t="n">
@@ -19350,7 +19350,7 @@
       </c>
       <c r="B768" t="inlineStr">
         <is>
-          <t>Sikander Azam</t>
+          <t>Fakhra Ghafoor</t>
         </is>
       </c>
       <c r="C768" t="n">
@@ -19371,7 +19371,7 @@
       </c>
       <c r="B769" t="inlineStr">
         <is>
-          <t>Fakhra Ghafoor</t>
+          <t>Bakhtiar Ul Haq</t>
         </is>
       </c>
       <c r="C769" t="n">
@@ -19392,7 +19392,7 @@
       </c>
       <c r="B770" t="inlineStr">
         <is>
-          <t>Muhammad Waqas</t>
+          <t>H W Seo</t>
         </is>
       </c>
       <c r="C770" t="n">
@@ -19413,7 +19413,7 @@
       </c>
       <c r="B771" t="inlineStr">
         <is>
-          <t>Abdul Shakoor</t>
+          <t>Muhammad Waqas</t>
         </is>
       </c>
       <c r="C771" t="n">
@@ -19434,7 +19434,7 @@
       </c>
       <c r="B772" t="inlineStr">
         <is>
-          <t>H W Seo</t>
+          <t>Sikander Azam</t>
         </is>
       </c>
       <c r="C772" t="n">
@@ -19539,7 +19539,7 @@
       </c>
       <c r="B777" t="inlineStr">
         <is>
-          <t>Yijun Shi</t>
+          <t>Jahan Zeb Gul</t>
         </is>
       </c>
       <c r="C777" t="n">
@@ -19560,7 +19560,7 @@
       </c>
       <c r="B778" t="inlineStr">
         <is>
-          <t>Yarjan Abdul Samad</t>
+          <t>Rayyan Ali Shaukat</t>
         </is>
       </c>
       <c r="C778" t="n">
@@ -19581,7 +19581,7 @@
       </c>
       <c r="B779" t="inlineStr">
         <is>
-          <t>Jahan Zeb Gul</t>
+          <t>Yarjan Abdul Samad</t>
         </is>
       </c>
       <c r="C779" t="n">
@@ -19602,7 +19602,7 @@
       </c>
       <c r="B780" t="inlineStr">
         <is>
-          <t>Rayyan Ali Shaukat</t>
+          <t>Yijun Shi</t>
         </is>
       </c>
       <c r="C780" t="n">
@@ -19644,7 +19644,7 @@
       </c>
       <c r="B782" t="inlineStr">
         <is>
-          <t>Ahmed Usman Ali</t>
+          <t>Ghayas Uddin Siddiqui</t>
         </is>
       </c>
       <c r="C782" t="n">
@@ -19665,7 +19665,7 @@
       </c>
       <c r="B783" t="inlineStr">
         <is>
-          <t>Ghayas Uddin Siddiqui</t>
+          <t>Ahmed Usman Ali</t>
         </is>
       </c>
       <c r="C783" t="n">
@@ -19749,7 +19749,7 @@
       </c>
       <c r="B787" t="inlineStr">
         <is>
-          <t>Anzar Mahmood</t>
+          <t>Bernabe Mari</t>
         </is>
       </c>
       <c r="C787" t="n">
@@ -19791,7 +19791,7 @@
       </c>
       <c r="B789" t="inlineStr">
         <is>
-          <t>Bernabe Mari</t>
+          <t>Anzar Mahmood</t>
         </is>
       </c>
       <c r="C789" t="n">
@@ -20085,7 +20085,7 @@
       </c>
       <c r="B803" t="inlineStr">
         <is>
-          <t>Muhammad Talha Amin</t>
+          <t>Faheem Khuhawar</t>
         </is>
       </c>
       <c r="C803" t="n">
@@ -20106,7 +20106,7 @@
       </c>
       <c r="B804" t="inlineStr">
         <is>
-          <t>Hafsa Shaikh</t>
+          <t>Muhammad Talha Amin</t>
         </is>
       </c>
       <c r="C804" t="n">
@@ -20127,7 +20127,7 @@
       </c>
       <c r="B805" t="inlineStr">
         <is>
-          <t>Faheem Khuhawar</t>
+          <t>Hafsa Shaikh</t>
         </is>
       </c>
       <c r="C805" t="n">
@@ -20148,7 +20148,7 @@
       </c>
       <c r="B806" t="inlineStr">
         <is>
-          <t>Sadia Ramzan</t>
+          <t>Tehmina Kalsum</t>
         </is>
       </c>
       <c r="C806" t="n">
@@ -20169,7 +20169,7 @@
       </c>
       <c r="B807" t="inlineStr">
         <is>
-          <t>Hafiz Arslan Ramzan</t>
+          <t>Sadia Ramzan</t>
         </is>
       </c>
       <c r="C807" t="n">
@@ -20190,7 +20190,7 @@
       </c>
       <c r="B808" t="inlineStr">
         <is>
-          <t>Tehmina Kalsum</t>
+          <t>Hafiz Arslan Ramzan</t>
         </is>
       </c>
       <c r="C808" t="n">
@@ -20547,7 +20547,7 @@
       </c>
       <c r="B825" t="inlineStr">
         <is>
-          <t>Samet Akcay</t>
+          <t>Naoufel Werghi</t>
         </is>
       </c>
       <c r="C825" t="n">
@@ -20568,7 +20568,7 @@
       </c>
       <c r="B826" t="inlineStr">
         <is>
-          <t>Naoufel Werghi</t>
+          <t>Samet Akcay</t>
         </is>
       </c>
       <c r="C826" t="n">
@@ -20589,7 +20589,7 @@
       </c>
       <c r="B827" t="inlineStr">
         <is>
-          <t>Aisha Gul Hafeez</t>
+          <t>Muhammad Shahzad</t>
         </is>
       </c>
       <c r="C827" t="n">
@@ -20610,7 +20610,7 @@
       </c>
       <c r="B828" t="inlineStr">
         <is>
-          <t>Muhammad Shahzad</t>
+          <t>Aisha Gul Hafeez</t>
         </is>
       </c>
       <c r="C828" t="n">
@@ -20736,7 +20736,7 @@
       </c>
       <c r="B834" t="inlineStr">
         <is>
-          <t>Imran Farid Nizami</t>
+          <t>Mobeen Ur Rahman</t>
         </is>
       </c>
       <c r="C834" t="n">
@@ -20757,7 +20757,7 @@
       </c>
       <c r="B835" t="inlineStr">
         <is>
-          <t>Mobeen Ur Rahman</t>
+          <t>Imran Farid Nizami</t>
         </is>
       </c>
       <c r="C835" t="n">
@@ -20862,7 +20862,7 @@
       </c>
       <c r="B840" t="inlineStr">
         <is>
-          <t>Aitzaz Saleem</t>
+          <t>Hassan Kazmi</t>
         </is>
       </c>
       <c r="C840" t="n">
@@ -20883,7 +20883,7 @@
       </c>
       <c r="B841" t="inlineStr">
         <is>
-          <t>Maheen Khalid</t>
+          <t>Aitzaz Saleem</t>
         </is>
       </c>
       <c r="C841" t="n">
@@ -20904,7 +20904,7 @@
       </c>
       <c r="B842" t="inlineStr">
         <is>
-          <t>Hassan Kazmi</t>
+          <t>Maheen Khalid</t>
         </is>
       </c>
       <c r="C842" t="n">
@@ -20946,7 +20946,7 @@
       </c>
       <c r="B844" t="inlineStr">
         <is>
-          <t>Ahmed</t>
+          <t>Abdelfatah Hassan</t>
         </is>
       </c>
       <c r="C844" t="n">
@@ -20967,7 +20967,7 @@
       </c>
       <c r="B845" t="inlineStr">
         <is>
-          <t>Abdelfatah Hassan</t>
+          <t>Ahmed</t>
         </is>
       </c>
       <c r="C845" t="n">
@@ -21009,7 +21009,7 @@
       </c>
       <c r="B847" t="inlineStr">
         <is>
-          <t>Jahan Zeb</t>
+          <t>Soyiba Jawed</t>
         </is>
       </c>
       <c r="C847" t="n">
@@ -21030,7 +21030,7 @@
       </c>
       <c r="B848" t="inlineStr">
         <is>
-          <t>Soyiba Jawed</t>
+          <t>Jahan Zeb</t>
         </is>
       </c>
       <c r="C848" t="n">
@@ -21051,7 +21051,7 @@
       </c>
       <c r="B849" t="inlineStr">
         <is>
-          <t>Asad Mansoor Khan</t>
+          <t>Muhammad Belal Afsar Khan</t>
         </is>
       </c>
       <c r="C849" t="n">
@@ -21072,7 +21072,7 @@
       </c>
       <c r="B850" t="inlineStr">
         <is>
-          <t>Muhammad Belal Afsar Khan</t>
+          <t>Asad Mansoor Khan</t>
         </is>
       </c>
       <c r="C850" t="n">
@@ -21135,7 +21135,7 @@
       </c>
       <c r="B853" t="inlineStr">
         <is>
-          <t>Syed Muhammad Anwar</t>
+          <t>Khawar Khurshid</t>
         </is>
       </c>
       <c r="C853" t="n">
@@ -21156,7 +21156,7 @@
       </c>
       <c r="B854" t="inlineStr">
         <is>
-          <t>Muhammad Majid</t>
+          <t>Imran Fareed Nizami</t>
         </is>
       </c>
       <c r="C854" t="n">
@@ -21177,7 +21177,7 @@
       </c>
       <c r="B855" t="inlineStr">
         <is>
-          <t>Khawar Khurshid</t>
+          <t>Mobeen Ur Rehman</t>
         </is>
       </c>
       <c r="C855" t="n">
@@ -21198,7 +21198,7 @@
       </c>
       <c r="B856" t="inlineStr">
         <is>
-          <t>Mobeen Ur Rehman</t>
+          <t>Syed Muhammad Anwar</t>
         </is>
       </c>
       <c r="C856" t="n">
@@ -21219,7 +21219,7 @@
       </c>
       <c r="B857" t="inlineStr">
         <is>
-          <t>Imran Fareed Nizami</t>
+          <t>Muhammad Majid</t>
         </is>
       </c>
       <c r="C857" t="n">
@@ -21240,7 +21240,7 @@
       </c>
       <c r="B858" t="inlineStr">
         <is>
-          <t>And Muhammad Usman Akram</t>
+          <t>Arslan Shaukat</t>
         </is>
       </c>
       <c r="C858" t="n">
@@ -21261,7 +21261,7 @@
       </c>
       <c r="B859" t="inlineStr">
         <is>
-          <t>Arslan Shaukat</t>
+          <t>Anum Abdus Salam</t>
         </is>
       </c>
       <c r="C859" t="n">
@@ -21282,7 +21282,7 @@
       </c>
       <c r="B860" t="inlineStr">
         <is>
-          <t>Anum Abdus Salam</t>
+          <t>And Muhammad Usman Akram</t>
         </is>
       </c>
       <c r="C860" t="n">
@@ -21303,7 +21303,7 @@
       </c>
       <c r="B861" t="inlineStr">
         <is>
-          <t>Mahboob Anwar</t>
+          <t>Mohammed Ghazal</t>
         </is>
       </c>
       <c r="C861" t="n">
@@ -21324,7 +21324,7 @@
       </c>
       <c r="B862" t="inlineStr">
         <is>
-          <t>Muhammad Owais</t>
+          <t>Mahboob Anwar</t>
         </is>
       </c>
       <c r="C862" t="n">
@@ -21345,7 +21345,7 @@
       </c>
       <c r="B863" t="inlineStr">
         <is>
-          <t>Mohammed Ghazal</t>
+          <t>Muhammad Owais</t>
         </is>
       </c>
       <c r="C863" t="n">

</xml_diff>

<commit_message>
fix: resolve LLM API key issue and add load_dotenv to all entry points
- Fix .env duplicate OPENAI_API_KEY (placeholder was shadowing real Groq key)
- Add load_dotenv(override=True) to pipeline_orchestrator.py before analysis imports
- Add load_dotenv(override=True) to api/main.py before FastAPI app init
- Add load_dotenv(override=True) to run_backend.py before uvicorn startup
- Add load_dotenv(override=True) to test_backend_api.py before all imports
- Read OPENAI_MODEL from env var in MasterPipeline (was hardcoded)

Result: 0 LLM 401 errors (was 43), all 58 tests pass including live Groq calls
</commit_message>
<xml_diff>
--- a/data/analysis/collaboration_profiles.xlsx
+++ b/data/analysis/collaboration_profiles.xlsx
@@ -618,12 +618,12 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>[{"name": "Roberto Quasso", "paper_count": 2}, {"name": "Luciano Lavagno", "paper_count": 2}, {"name": "Mihai T Lazarescu", "paper_count": 2}]</t>
+          <t>[{"name": "Luciano Lavagno", "paper_count": 2}, {"name": "Roberto Quasso", "paper_count": 2}, {"name": "Mihai T Lazarescu", "paper_count": 2}]</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Candidate Nasir Ali Shah has collaborated with 14 unique co-author(s) across 4 publication(s). They operate as a Large-Group Researcher with an average of 5.2 authors per paper. The candidate has 3 recurring collaborator(s) (top co-authors: Roberto Quasso (2 papers), Luciano Lavagno (2 papers), Mihai T Lazarescu (2 papers)). Overall research collaboration network is categorized as Broad Network.</t>
+          <t>Candidate Nasir Ali Shah has collaborated with 14 unique co-author(s) across 4 publication(s). They operate as a Large-Group Researcher with an average of 5.2 authors per paper. The candidate has 3 recurring collaborator(s) (top co-authors: Luciano Lavagno (2 papers), Roberto Quasso (2 papers), Mihai T Lazarescu (2 papers)). Overall research collaboration network is categorized as Broad Network.</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -744,12 +744,12 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>[{"name": "Tayyaba Gul Tareen", "paper_count": 4}, {"name": "Muhammad Aamir", "paper_count": 2}, {"name": "Jehanzeb Khan", "paper_count": 2}]</t>
+          <t>[{"name": "Tayyaba Gul Tareen", "paper_count": 4}, {"name": "Jehanzeb Khan", "paper_count": 2}, {"name": "Muhammad Aamir", "paper_count": 2}]</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Candidate Tayyaba Gull has collaborated with 13 unique co-author(s) across 5 publication(s). They operate as a Medium-Group Researcher with an average of 4.6 authors per paper. The candidate has 3 recurring collaborator(s) (top co-authors: Tayyaba Gul Tareen (4 papers), Muhammad Aamir (2 papers), Jehanzeb Khan (2 papers)). Overall research collaboration network is categorized as Broad Network.</t>
+          <t>Candidate Tayyaba Gull has collaborated with 13 unique co-author(s) across 5 publication(s). They operate as a Medium-Group Researcher with an average of 4.6 authors per paper. The candidate has 3 recurring collaborator(s) (top co-authors: Tayyaba Gul Tareen (4 papers), Jehanzeb Khan (2 papers), Muhammad Aamir (2 papers)). Overall research collaboration network is categorized as Broad Network.</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -933,12 +933,12 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>[{"name": "S Tamoor Ul Hassan", "paper_count": 6}, {"name": "M Latva Aho", "paper_count": 4}, {"name": "M Bennis", "paper_count": 4}, {"name": "Ashraf", "paper_count": 2}, {"name": "S Samarakoon", "paper_count": 2}]</t>
+          <t>[{"name": "S Tamoor Ul Hassan", "paper_count": 6}, {"name": "M Bennis", "paper_count": 4}, {"name": "M Latva Aho", "paper_count": 4}, {"name": "Ashraf", "paper_count": 2}, {"name": "S Samarakoon", "paper_count": 2}]</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Candidate SYED TAMOORULHASSAN has collaborated with 18 unique co-author(s) across 7 publication(s). They operate as a Large-Group Researcher with an average of 5.6 authors per paper. The candidate has 6 recurring collaborator(s) (top co-authors: S Tamoor Ul Hassan (6 papers), M Latva Aho (4 papers), M Bennis (4 papers)). Overall research collaboration network is categorized as Broad Network.</t>
+          <t>Candidate SYED TAMOORULHASSAN has collaborated with 18 unique co-author(s) across 7 publication(s). They operate as a Large-Group Researcher with an average of 5.6 authors per paper. The candidate has 6 recurring collaborator(s) (top co-authors: S Tamoor Ul Hassan (6 papers), M Bennis (4 papers), M Latva Aho (4 papers)). Overall research collaboration network is categorized as Broad Network.</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -996,7 +996,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>[{"name": "Waheed Aftab Khan", "paper_count": 5}, {"name": "W A Khan", "paper_count": 4}, {"name": "G Abbas", "paper_count": 4}, {"name": "Ali Raza", "paper_count": 3}, {"name": "Hafiz Fuad Usman", "paper_count": 3}]</t>
+          <t>[{"name": "Waheed Aftab Khan", "paper_count": 5}, {"name": "W A Khan", "paper_count": 4}, {"name": "G Abbas", "paper_count": 4}, {"name": "Hafiz Fuad Usman", "paper_count": 3}, {"name": "Ali Raza", "paper_count": 3}]</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1059,12 +1059,12 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>[{"name": "G Marchetto", "paper_count": 9}, {"name": "V Curri", "paper_count": 8}, {"name": "A Ahmad", "paper_count": 8}, {"name": "A Bianco", "paper_count": 8}, {"name": "H Chouman", "paper_count": 7}]</t>
+          <t>[{"name": "G Marchetto", "paper_count": 9}, {"name": "A Bianco", "paper_count": 8}, {"name": "A Ahmad", "paper_count": 8}, {"name": "V Curri", "paper_count": 8}, {"name": "H Chouman", "paper_count": 7}]</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Candidate Sarosh Tahir has collaborated with 16 unique co-author(s) across 10 publication(s). They operate as a Large-Group Researcher with an average of 6.2 authors per paper. The candidate has 6 recurring collaborator(s) (top co-authors: G Marchetto (9 papers), V Curri (8 papers), A Ahmad (8 papers)). Overall research collaboration network is categorized as Broad Network.</t>
+          <t>Candidate Sarosh Tahir has collaborated with 16 unique co-author(s) across 10 publication(s). They operate as a Large-Group Researcher with an average of 6.2 authors per paper. The candidate has 6 recurring collaborator(s) (top co-authors: G Marchetto (9 papers), A Bianco (8 papers), A Ahmad (8 papers)). Overall research collaboration network is categorized as Broad Network.</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
@@ -1122,12 +1122,12 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>[{"name": "Shakil Rehman", "paper_count": 3}, {"name": "Sheikh", "paper_count": 3}, {"name": "Shakil R Sheikh", "paper_count": 3}, {"name": "Noman Naseer", "paper_count": 3}, {"name": "Ghafoor", "paper_count": 2}]</t>
+          <t>[{"name": "Sheikh", "paper_count": 3}, {"name": "Shakil Rehman", "paper_count": 3}, {"name": "Shakil R Sheikh", "paper_count": 3}, {"name": "Noman Naseer", "paper_count": 3}, {"name": "Nouman", "paper_count": 2}]</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Candidate Muzzamil Ghaffar has collaborated with 23 unique co-author(s) across 6 publication(s). They operate as a Large-Group Researcher with an average of 6.7 authors per paper. The candidate has 7 recurring collaborator(s) (top co-authors: Shakil Rehman (3 papers), Sheikh (3 papers), Shakil R Sheikh (3 papers)). Overall research collaboration network is categorized as Broad Network.</t>
+          <t>Candidate Muzzamil Ghaffar has collaborated with 23 unique co-author(s) across 6 publication(s). They operate as a Large-Group Researcher with an average of 6.7 authors per paper. The candidate has 7 recurring collaborator(s) (top co-authors: Sheikh (3 papers), Shakil Rehman (3 papers), Shakil R Sheikh (3 papers)). Overall research collaboration network is categorized as Broad Network.</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
@@ -1185,12 +1185,12 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>[{"name": "Zz Abidin", "paper_count": 5}, {"name": "Kamarudin", "paper_count": 4}, {"name": "Ayi Ashyap", "paper_count": 3}, {"name": "Ha Majid", "paper_count": 3}, {"name": "Mh Dahri", "paper_count": 2}]</t>
+          <t>[{"name": "Zz Abidin", "paper_count": 5}, {"name": "Kamarudin", "paper_count": 4}, {"name": "Ha Majid", "paper_count": 3}, {"name": "Ayi Ashyap", "paper_count": 3}, {"name": "Mi Abbasi", "paper_count": 2}]</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Candidate Suhail Asghar Qureshi has collaborated with 23 unique co-author(s) across 8 publication(s). They operate as a Large-Group Researcher with an average of 5.8 authors per paper. The candidate has 7 recurring collaborator(s) (top co-authors: Zz Abidin (5 papers), Kamarudin (4 papers), Ayi Ashyap (3 papers)). Overall research collaboration network is categorized as Broad Network.</t>
+          <t>Candidate Suhail Asghar Qureshi has collaborated with 23 unique co-author(s) across 8 publication(s). They operate as a Large-Group Researcher with an average of 5.8 authors per paper. The candidate has 7 recurring collaborator(s) (top co-authors: Zz Abidin (5 papers), Kamarudin (4 papers), Ha Majid (3 papers)). Overall research collaboration network is categorized as Broad Network.</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
@@ -1437,12 +1437,12 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>[{"name": "Claus Pahl", "paper_count": 5}, {"name": "Waheed Ur Rehman", "paper_count": 3}, {"name": "Hamid R Barzegar", "paper_count": 3}, {"name": "Nabil El Ioini", "paper_count": 3}, {"name": "Ibe Van Thillo", "paper_count": 2}]</t>
+          <t>[{"name": "Claus Pahl", "paper_count": 5}, {"name": "Waheed Ur Rehman", "paper_count": 3}, {"name": "Nabil El Ioini", "paper_count": 3}, {"name": "Hamid R Barzegar", "paper_count": 3}, {"name": "Ibe Van Thillo", "paper_count": 2}]</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>Candidate Zeeshan has collaborated with 26 unique co-author(s) across 10 publication(s). They operate as a Large-Group Researcher with an average of 5.2 authors per paper. The candidate has 6 recurring collaborator(s) (top co-authors: Claus Pahl (5 papers), Waheed Ur Rehman (3 papers), Hamid R Barzegar (3 papers)). Overall research collaboration network is categorized as Broad Network.</t>
+          <t>Candidate Zeeshan has collaborated with 26 unique co-author(s) across 10 publication(s). They operate as a Large-Group Researcher with an average of 5.2 authors per paper. The candidate has 6 recurring collaborator(s) (top co-authors: Claus Pahl (5 papers), Waheed Ur Rehman (3 papers), Nabil El Ioini (3 papers)). Overall research collaboration network is categorized as Broad Network.</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
@@ -1500,12 +1500,12 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>[{"name": "Muhammad Saadi", "paper_count": 7}, {"name": "Hu Jin", "paper_count": 6}, {"name": "Jun Bae Seo", "paper_count": 6}, {"name": "Lunchakorn Wuttisittikulkij", "paper_count": 3}, {"name": "Saqib Ali Khan", "paper_count": 3}]</t>
+          <t>[{"name": "Muhammad Saadi", "paper_count": 7}, {"name": "Jun Bae Seo", "paper_count": 6}, {"name": "Hu Jin", "paper_count": 6}, {"name": "Lunchakorn Wuttisittikulkij", "paper_count": 3}, {"name": "Saqib Ali Khan", "paper_count": 3}]</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>Candidate Waqas Tariq Toor has collaborated with 83 unique co-author(s) across 29 publication(s). They operate as a Large-Group Researcher with an average of 5.1 authors per paper. The candidate has 15 recurring collaborator(s) (top co-authors: Muhammad Saadi (7 papers), Hu Jin (6 papers), Jun Bae Seo (6 papers)). Overall research collaboration network is categorized as Broad Network.</t>
+          <t>Candidate Waqas Tariq Toor has collaborated with 83 unique co-author(s) across 29 publication(s). They operate as a Large-Group Researcher with an average of 5.1 authors per paper. The candidate has 15 recurring collaborator(s) (top co-authors: Muhammad Saadi (7 papers), Jun Bae Seo (6 papers), Hu Jin (6 papers)). Overall research collaboration network is categorized as Broad Network.</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
@@ -1626,7 +1626,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>[{"name": "Danish Khan", "paper_count": 7}, {"name": "Manoj Kumar Panjwani", "paper_count": 4}, {"name": "Tahir Iqbal", "paper_count": 3}, {"name": "Honglu Zhu", "paper_count": 3}, {"name": "Chang Qing Dong", "paper_count": 2}]</t>
+          <t>[{"name": "Danish Khan", "paper_count": 7}, {"name": "Manoj Kumar Panjwani", "paper_count": 4}, {"name": "Tahir Iqbal", "paper_count": 3}, {"name": "Honglu Zhu", "paper_count": 3}, {"name": "Zafar Hussain", "paper_count": 2}]</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -1752,12 +1752,12 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>[{"name": "F S", "paper_count": 9}, {"name": "M", "paper_count": 6}, {"name": "Sugiyama", "paper_count": 5}, {"name": "K", "paper_count": 5}, {"name": "Fujii", "paper_count": 5}]</t>
+          <t>[{"name": "F S", "paper_count": 9}, {"name": "M", "paper_count": 6}, {"name": "Nakano", "paper_count": 5}, {"name": "K", "paper_count": 5}, {"name": "Sugiyama", "paper_count": 5}]</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>Candidate Fahd Sikandar Khan has collaborated with 32 unique co-author(s) across 9 publication(s). They operate as a Large-Group Researcher with an average of 9.0 authors per paper. The candidate has 10 recurring collaborator(s) (top co-authors: F S (9 papers), M (6 papers), Sugiyama (5 papers)). Overall research collaboration network is categorized as Broad Network.</t>
+          <t>Candidate Fahd Sikandar Khan has collaborated with 32 unique co-author(s) across 9 publication(s). They operate as a Large-Group Researcher with an average of 9.0 authors per paper. The candidate has 10 recurring collaborator(s) (top co-authors: F S (9 papers), M (6 papers), Nakano (5 papers)). Overall research collaboration network is categorized as Broad Network.</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
@@ -2382,12 +2382,12 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>[{"name": "Sobia Jangsher", "paper_count": 4}, {"name": "Ashfaq Ahmed", "paper_count": 2}, {"name": "Adnan Zafar", "paper_count": 2}]</t>
+          <t>[{"name": "Sobia Jangsher", "paper_count": 4}, {"name": "Adnan Zafar", "paper_count": 2}, {"name": "Ashfaq Ahmed", "paper_count": 2}]</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>Candidate Aamina Akbar has collaborated with 7 unique co-author(s) across 4 publication(s). They operate as a Medium-Group Researcher with an average of 4.0 authors per paper. The candidate has 3 recurring collaborator(s) (top co-authors: Sobia Jangsher (4 papers), Ashfaq Ahmed (2 papers), Adnan Zafar (2 papers)). Overall research collaboration network is categorized as Balanced Network.</t>
+          <t>Candidate Aamina Akbar has collaborated with 7 unique co-author(s) across 4 publication(s). They operate as a Medium-Group Researcher with an average of 4.0 authors per paper. The candidate has 3 recurring collaborator(s) (top co-authors: Sobia Jangsher (4 papers), Adnan Zafar (2 papers), Ashfaq Ahmed (2 papers)). Overall research collaboration network is categorized as Balanced Network.</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
@@ -2445,7 +2445,7 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>[{"name": "Syed Ali Hassan", "paper_count": 7}, {"name": "Shah Zeb", "paper_count": 4}, {"name": "Mikael Gidlund", "paper_count": 2}, {"name": "Aamir Mahmood", "paper_count": 2}, {"name": "Syed Ali Raza Zaidi", "paper_count": 2}]</t>
+          <t>[{"name": "Syed Ali Hassan", "paper_count": 7}, {"name": "Shah Zeb", "paper_count": 4}, {"name": "Mikael Gidlund", "paper_count": 2}, {"name": "Aamir Mahmood", "paper_count": 2}, {"name": "Rafia Mumtaz", "paper_count": 2}]</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
@@ -2508,12 +2508,12 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>[{"name": "Eun Sung Jung", "paper_count": 5}, {"name": "Hyung Seok Kim", "paper_count": 5}, {"name": "Rashid Ali", "paper_count": 4}, {"name": "Amir Haider", "paper_count": 4}, {"name": "M Zubair Islam", "paper_count": 2}]</t>
+          <t>[{"name": "Eun Sung Jung", "paper_count": 5}, {"name": "Hyung Seok Kim", "paper_count": 5}, {"name": "Amir Haider", "paper_count": 4}, {"name": "Rashid Ali", "paper_count": 4}, {"name": "M Zubair Islam", "paper_count": 2}]</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>Candidate Shahzad has collaborated with 8 unique co-author(s) across 9 publication(s). They operate as a Medium-Group Researcher with an average of 3.6 authors per paper. The candidate has 5 recurring collaborator(s) (top co-authors: Eun Sung Jung (5 papers), Hyung Seok Kim (5 papers), Rashid Ali (4 papers)). Overall research collaboration network is categorized as Balanced Network.</t>
+          <t>Candidate Shahzad has collaborated with 8 unique co-author(s) across 9 publication(s). They operate as a Medium-Group Researcher with an average of 3.6 authors per paper. The candidate has 5 recurring collaborator(s) (top co-authors: Eun Sung Jung (5 papers), Hyung Seok Kim (5 papers), Amir Haider (4 papers)). Overall research collaboration network is categorized as Balanced Network.</t>
         </is>
       </c>
       <c r="O33" t="inlineStr">
@@ -3348,7 +3348,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Shanshan Tu</t>
+          <t>Fazal Muhammad</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -3369,7 +3369,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Asar Ali</t>
+          <t>Ammar Armghan</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -3390,7 +3390,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Ammar Armghan</t>
+          <t>Fayadh Alenezi</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -3411,7 +3411,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Norah Alnaim</t>
+          <t>Farman Ali</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -3432,7 +3432,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Farman Ali</t>
+          <t>Shanshan Tu</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -3453,7 +3453,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Fazal Muhammad</t>
+          <t>Asar Ali</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -3474,7 +3474,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Fayadh Alenezi</t>
+          <t>Norah Alnaim</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -3537,7 +3537,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Amil Daraz</t>
+          <t>Salman A Alqahtani</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -3558,7 +3558,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Atif M Alamri</t>
+          <t>Amil Daraz</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -3579,7 +3579,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Salman A Alqahtani</t>
+          <t>Atif M Alamri</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -3600,7 +3600,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Roberto Quasso</t>
+          <t>Luciano Lavagno</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -3621,7 +3621,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Luciano Lavagno</t>
+          <t>Roberto Quasso</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -3663,7 +3663,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Ghulam E Mustafa Abro</t>
+          <t>Abdinasir Hirsi</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -3705,7 +3705,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Ardhi Wijayanto</t>
+          <t>Abdul Rehman Altaf</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3726,7 +3726,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Abdinasir Hirsi</t>
+          <t>Nabihah Ahmad</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3747,7 +3747,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Nabihah Ahmad</t>
+          <t>Ghulam E Mustafa Abro</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3768,7 +3768,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Abdul Rehman Altaf</t>
+          <t>Ardhi Wijayanto</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3789,7 +3789,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Syed Tahir Hussain Rizvi</t>
+          <t>Achraf Jabeur Telmoudi</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3831,7 +3831,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Achraf Jabeur Telmoudi</t>
+          <t>Muhammad Yasir Latif</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3852,7 +3852,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Muhammad Yasir Latif</t>
+          <t>Syed Tahir Hussain Rizvi</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -4062,7 +4062,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Mohammed A Al Masni</t>
+          <t>Nagwan Abdel Samee</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -4083,7 +4083,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Nagwan Abdel Samee</t>
+          <t>Mohammed A Al Masni</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -4209,7 +4209,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Syeda Javeria Ahsan</t>
+          <t>Rahmat Ullah</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -4251,7 +4251,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Mujeeb Ur Rehman</t>
+          <t>Syeda Javeria Ahsan</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -4272,7 +4272,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Rahmat Ullah</t>
+          <t>Mujeeb Ur Rehman</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -4314,7 +4314,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Arsalan Khurshid</t>
+          <t>Hafza Ayesha Siddiqa</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -4335,7 +4335,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Saadullah Farooq Abbasi</t>
+          <t>Chen Chen</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -4356,7 +4356,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Yan Xu</t>
+          <t>Laishuan Wang</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -4377,7 +4377,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Chen Chen</t>
+          <t>Arsalan Khurshid</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -4398,7 +4398,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Wei Chen</t>
+          <t>Yan Xu</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -4419,7 +4419,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Hafza Ayesha Siddiqa</t>
+          <t>Wei Chen</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -4440,7 +4440,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Laishuan Wang</t>
+          <t>Saadullah Farooq Abbasi</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -4461,7 +4461,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Zhuangzhuang Du</t>
+          <t>Hafiz Abbad Ur Rehman</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -4482,7 +4482,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Hafiz Abbad Ur Rehman</t>
+          <t>Zhuangzhuang Du</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -4524,7 +4524,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Ali Imran</t>
+          <t>Hussain Al Faisal</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -4545,7 +4545,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Hussain Al Faisal</t>
+          <t>Ali Imran</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -4608,7 +4608,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Muhammad Armghan Latif</t>
+          <t>Maali Alabdulhafith</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -4629,7 +4629,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Sara Rehman</t>
+          <t>Muhammad Armghan Latif</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -4650,7 +4650,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Maali Alabdulhafith</t>
+          <t>Sara Rehman</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -4671,7 +4671,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Yeong Hyeon Gu</t>
+          <t>Hafiz Ghulam Murtza Qamar</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -4713,7 +4713,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Hafiz Ghulam Murtza Qamar</t>
+          <t>Yeong Hyeon Gu</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -4776,7 +4776,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Sabtain Raza</t>
+          <t>Muhammad Taha</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -4797,7 +4797,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Muhammad Taha</t>
+          <t>Sabtain Raza</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -4818,7 +4818,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Qamar Akhter</t>
+          <t>Paranav Kumar Pathak</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -4839,7 +4839,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Abubakar Siddique</t>
+          <t>Qamar Akhter</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -4860,7 +4860,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Salman A Alqahtani</t>
+          <t>Waseem Aslam</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -4881,7 +4881,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Paranav Kumar Pathak</t>
+          <t>Abubakar Siddique</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -4923,7 +4923,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Waseem Aslam</t>
+          <t>Salman A Alqahtani</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -4965,7 +4965,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Abdul Quddoos Sabeeh</t>
+          <t>Abid Mushtaq</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -5049,7 +5049,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Abid Mushtaq</t>
+          <t>Abdul Quddoos Sabeeh</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -5070,7 +5070,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Uroosa Nawaz</t>
+          <t>Saman Khalil</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -5091,7 +5091,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Khalid Alhussaini</t>
+          <t>Adham Aleid</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -5112,7 +5112,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Saman Khalil</t>
+          <t>Khalid Alhussaini</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -5133,7 +5133,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Abdul Malik</t>
+          <t>Uroosa Nawaz</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -5154,7 +5154,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Adham Aleid</t>
+          <t>Abdul Malik</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -5196,7 +5196,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Imran Siddique</t>
+          <t>Nabeel Ahmed Khan</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -5238,7 +5238,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Nabeel Ahmed Khan</t>
+          <t>Imran Siddique</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -5343,7 +5343,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Arsalan Habib</t>
+          <t>Thierry</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -5364,7 +5364,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Khawaja</t>
+          <t>Olivier D</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -5385,7 +5385,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Bernal</t>
+          <t>Saqib</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -5406,7 +5406,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Usman</t>
+          <t>Zabit</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -5427,7 +5427,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Thierry</t>
+          <t>Bernal</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -5448,7 +5448,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Bosch</t>
+          <t>Khawaja</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -5469,7 +5469,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Amin</t>
+          <t>Usman</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -5490,7 +5490,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Saqib</t>
+          <t>Amin</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -5511,7 +5511,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Zabit</t>
+          <t>Bosch</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -5532,7 +5532,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Olivier D</t>
+          <t>Arsalan Habib</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -5574,7 +5574,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Rehman</t>
+          <t>Muhammad Ziaur</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -5595,7 +5595,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Muhammad Ziaur</t>
+          <t>Rehman</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -5868,7 +5868,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Serestina Viriri</t>
+          <t>Umber Saba</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -5889,7 +5889,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Umber Saba</t>
+          <t>Serestina Viriri</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -5952,7 +5952,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Muhammad Aamir</t>
+          <t>Jehanzeb Khan</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -5973,7 +5973,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Jehanzeb Khan</t>
+          <t>Muhammad Aamir</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -6057,7 +6057,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Mehr E Munir</t>
+          <t>Shahryar Shafique</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -6078,7 +6078,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Shahryar Shafique</t>
+          <t>Mehr E Munir</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -6099,7 +6099,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Tayyaba Tareen</t>
+          <t>Nasir Saleem</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -6120,7 +6120,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Nasir Saleem</t>
+          <t>Tayyaba Tareen</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -6330,7 +6330,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>Khalid Masood</t>
+          <t>Muhammad Faheem</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -6351,7 +6351,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Muhammad Faheem</t>
+          <t>Khalid Masood</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -6372,7 +6372,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>Bo Wang</t>
+          <t>Khalil Ur Rehman</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -6393,7 +6393,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>Khalil Ur Rehman</t>
+          <t>Bo Wang</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -6435,7 +6435,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>Yue Shen</t>
+          <t>Liu Hui</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -6456,7 +6456,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>Liu Hui</t>
+          <t>Yue Shen</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -6561,7 +6561,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>Saima Yousaf</t>
+          <t>Faiza Rehman</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -6582,7 +6582,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>Faiza Rehman</t>
+          <t>Saima Yousaf</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -6624,7 +6624,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>Saba Mohsin</t>
+          <t>Syeda Urwa Warsi</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -6666,7 +6666,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>Syeda Urwa Warsi</t>
+          <t>Saba Mohsin</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -6687,7 +6687,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>Masood</t>
+          <t>Muhammad Khalid Mudassar</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -6708,7 +6708,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>Muhammad Khalid Mudassar</t>
+          <t>Masood</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -6750,7 +6750,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>Amber Sultan</t>
+          <t>Hanan Sharif</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -6771,7 +6771,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>Hanan Sharif</t>
+          <t>Amber Sultan</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -6834,7 +6834,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>Muhammad Arfan Ali Nagra</t>
+          <t>Muhammad Sohail</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -6855,7 +6855,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>Muhammad Sohail</t>
+          <t>Muhammad Arfan Ali Nagra</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -6939,7 +6939,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>Muhammad Naeem Aslam</t>
+          <t>Alghamdi</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -6960,7 +6960,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>Alghamdi</t>
+          <t>Muhammad Naeem Aslam</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -6981,7 +6981,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>Ahmad Alshammari</t>
+          <t>Muhammad Ahsan Raza</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -7023,7 +7023,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>Anas Bilal</t>
+          <t>Ahmad Alshammari</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -7044,7 +7044,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>Muhammad Ahsan Raza</t>
+          <t>Anas Bilal</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -7065,7 +7065,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>Muhammad Irfan</t>
+          <t>Tomasz Jakubowski</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -7086,7 +7086,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>Nabeel Ahmed</t>
+          <t>Saifur Rahman Khan</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -7107,7 +7107,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>Paweł Sokołowski</t>
+          <t>Muhammad Irfan</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -7128,7 +7128,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>Zohaib Mushtaq</t>
+          <t>Paweł Sokołowski</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -7149,7 +7149,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>Tomasz Jakubowski</t>
+          <t>Nabeel Ahmed</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -7170,7 +7170,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>Grzegorz Nawalany</t>
+          <t>Zohaib Mushtaq</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -7191,7 +7191,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>Saifur Rahman Khan</t>
+          <t>Grzegorz Nawalany</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -7212,7 +7212,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>Muhammad Nadeem</t>
+          <t>Mi Kyung Park</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -7233,7 +7233,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>Mi Kyung Park</t>
+          <t>Saqib Ameer</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -7338,7 +7338,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>Saqib Ameer</t>
+          <t>Muhammad Nadeem</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -7359,7 +7359,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>Xiang Lin Zhu</t>
+          <t>Muhammad Ajmal</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -7401,7 +7401,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>Muhammad Ajmal</t>
+          <t>Xiang Lin Zhu</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -7422,7 +7422,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>Noor Rehman</t>
+          <t>Talal Ahmad</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -7464,7 +7464,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>Talal Ahmad</t>
+          <t>Noor Rehman</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -7548,7 +7548,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>Ling Qh</t>
+          <t>Mehta S</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -7569,7 +7569,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>Mehta S</t>
+          <t>Han F</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -7590,7 +7590,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>Han F</t>
+          <t>Ling Qh</t>
         </is>
       </c>
       <c r="C208" t="n">
@@ -7611,7 +7611,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>Nagra Aa</t>
+          <t>Apasiba At</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -7632,7 +7632,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>Apasiba At</t>
+          <t>Nagra Aa</t>
         </is>
       </c>
       <c r="C210" t="n">
@@ -7674,7 +7674,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>Haris Jawad Arain</t>
+          <t>Sheikh Junaid Yawar</t>
         </is>
       </c>
       <c r="C212" t="n">
@@ -7695,7 +7695,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>Sheikh Junaid Yawar</t>
+          <t>Haris Jawad Arain</t>
         </is>
       </c>
       <c r="C213" t="n">
@@ -7737,7 +7737,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>Xianglin Zhu</t>
+          <t>Muhammad Ashfaq</t>
         </is>
       </c>
       <c r="C215" t="n">
@@ -7758,7 +7758,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>Muhammad Ashfaq</t>
+          <t>Xianglin Zhu</t>
         </is>
       </c>
       <c r="C216" t="n">
@@ -7779,7 +7779,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>Aamir Nazir</t>
+          <t>Sheeraz Arif</t>
         </is>
       </c>
       <c r="C217" t="n">
@@ -7800,7 +7800,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>Sheeraz Arif</t>
+          <t>Aamir Nazir</t>
         </is>
       </c>
       <c r="C218" t="n">
@@ -7968,7 +7968,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>Qihuang</t>
+          <t>Khalidumer</t>
         </is>
       </c>
       <c r="C226" t="n">
@@ -7989,7 +7989,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>Khalidumer</t>
+          <t>Qihuang</t>
         </is>
       </c>
       <c r="C227" t="n">
@@ -8115,7 +8115,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>Muhammad Husnain Haider</t>
+          <t>Fazal Hussain</t>
         </is>
       </c>
       <c r="C233" t="n">
@@ -8136,7 +8136,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>Fazal Hussain</t>
+          <t>Muhammad Husnain Haider</t>
         </is>
       </c>
       <c r="C234" t="n">
@@ -8157,7 +8157,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>Hassam Ishfaq</t>
+          <t>Mubarak Abdussalam</t>
         </is>
       </c>
       <c r="C235" t="n">
@@ -8178,7 +8178,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>Mubarak Abdussalam</t>
+          <t>Hassam Ishfaq</t>
         </is>
       </c>
       <c r="C236" t="n">
@@ -8241,7 +8241,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>Umashankar Subramaniam</t>
+          <t>Sivakumar Selvam</t>
         </is>
       </c>
       <c r="C239" t="n">
@@ -8262,7 +8262,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>Sivakumar Selvam</t>
+          <t>Umashankar Subramaniam</t>
         </is>
       </c>
       <c r="C240" t="n">
@@ -8325,7 +8325,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>M Naeem</t>
+          <t>K Umer</t>
         </is>
       </c>
       <c r="C243" t="n">
@@ -8367,7 +8367,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>K Umer</t>
+          <t>M Naeem</t>
         </is>
       </c>
       <c r="C245" t="n">
@@ -8388,7 +8388,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>Syed Adreesahmed</t>
+          <t>Zhenyuanzhang</t>
         </is>
       </c>
       <c r="C246" t="n">
@@ -8409,7 +8409,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>Zhenyuanzhang</t>
+          <t>Syed Adreesahmed</t>
         </is>
       </c>
       <c r="C247" t="n">
@@ -8430,7 +8430,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>Muhammadafzal</t>
+          <t>Syed Adreesahmad</t>
         </is>
       </c>
       <c r="C248" t="n">
@@ -8451,7 +8451,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>Syed Adreesahmad</t>
+          <t>Muhammadafzal</t>
         </is>
       </c>
       <c r="C249" t="n">
@@ -8493,7 +8493,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>Ateeq</t>
+          <t>Khawaja Wajiha</t>
         </is>
       </c>
       <c r="C251" t="n">
@@ -8535,7 +8535,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>Khawaja Wajiha</t>
+          <t>Ateeq</t>
         </is>
       </c>
       <c r="C253" t="n">
@@ -8577,7 +8577,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>Khwaja Mutahir Ahmad</t>
+          <t>Rajesh Kumar</t>
         </is>
       </c>
       <c r="C255" t="n">
@@ -8598,7 +8598,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>Rajesh Kumar</t>
+          <t>Khwaja Mutahir Ahmad</t>
         </is>
       </c>
       <c r="C256" t="n">
@@ -8787,7 +8787,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>Kola Narasimha</t>
+          <t>Sarathbabu</t>
         </is>
       </c>
       <c r="C265" t="n">
@@ -8808,7 +8808,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>Sarathbabu</t>
+          <t>Raju</t>
         </is>
       </c>
       <c r="C266" t="n">
@@ -8829,7 +8829,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>Raju</t>
+          <t>Kola Narasimha</t>
         </is>
       </c>
       <c r="C267" t="n">
@@ -8955,7 +8955,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>Mahnoorshahzadi</t>
+          <t>Foo Yi Shyheddy</t>
         </is>
       </c>
       <c r="C273" t="n">
@@ -8997,7 +8997,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>Foo Yi Shyheddy</t>
+          <t>Mahnoorshahzadi</t>
         </is>
       </c>
       <c r="C275" t="n">
@@ -9039,7 +9039,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>M Latva Aho</t>
+          <t>M Bennis</t>
         </is>
       </c>
       <c r="C277" t="n">
@@ -9060,7 +9060,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>M Bennis</t>
+          <t>M Latva Aho</t>
         </is>
       </c>
       <c r="C278" t="n">
@@ -9144,7 +9144,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>H Bagheri</t>
+          <t>Marcos Katz</t>
         </is>
       </c>
       <c r="C282" t="n">
@@ -9165,7 +9165,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>M Ikram</t>
+          <t>H Chowdhury</t>
         </is>
       </c>
       <c r="C283" t="n">
@@ -9186,7 +9186,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>H Chowdhury</t>
+          <t>H Bagheri</t>
         </is>
       </c>
       <c r="C284" t="n">
@@ -9207,7 +9207,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>Marcos Katz</t>
+          <t>M Ikram</t>
         </is>
       </c>
       <c r="C285" t="n">
@@ -9249,7 +9249,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>Syed Tamoor Ul Hassan</t>
+          <t>Shahid Mumtaz</t>
         </is>
       </c>
       <c r="C287" t="n">
@@ -9270,7 +9270,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>Kim Fung Tsang</t>
+          <t>Muhammad Ikram</t>
         </is>
       </c>
       <c r="C288" t="n">
@@ -9291,7 +9291,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>Muhammad Ikram</t>
+          <t>Syed Tamoor Ul Hassan</t>
         </is>
       </c>
       <c r="C289" t="n">
@@ -9312,7 +9312,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>Shahid Mumtaz</t>
+          <t>Kim Fung Tsang</t>
         </is>
       </c>
       <c r="C290" t="n">
@@ -9459,7 +9459,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>Ali Raza</t>
+          <t>Hafiz Fuad Usman</t>
         </is>
       </c>
       <c r="C297" t="n">
@@ -9480,7 +9480,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>Hafiz Fuad Usman</t>
+          <t>Ali Raza</t>
         </is>
       </c>
       <c r="C298" t="n">
@@ -9711,7 +9711,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Muhammad Numan Khan</t>
+          <t>Muhammad Waqar Hassan</t>
         </is>
       </c>
       <c r="C309" t="n">
@@ -9732,7 +9732,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Muhammad Waqar Hassan</t>
+          <t>Muhammad Numan Khan</t>
         </is>
       </c>
       <c r="C310" t="n">
@@ -9753,7 +9753,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Waheed A Khan</t>
+          <t>Kamran Daniel</t>
         </is>
       </c>
       <c r="C311" t="n">
@@ -9774,7 +9774,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Noman Shabbir</t>
+          <t>Waheed A Khan</t>
         </is>
       </c>
       <c r="C312" t="n">
@@ -9795,7 +9795,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Muhammad Rehan Usman</t>
+          <t>Noman Shabbir</t>
         </is>
       </c>
       <c r="C313" t="n">
@@ -9816,7 +9816,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Kamran Daniel</t>
+          <t>Gandeva Bayu Satrya</t>
         </is>
       </c>
       <c r="C314" t="n">
@@ -9837,7 +9837,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Gandeva Bayu Satrya</t>
+          <t>Muhammad Rehan Usman</t>
         </is>
       </c>
       <c r="C315" t="n">
@@ -9858,7 +9858,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Nouman Ali</t>
+          <t>Umair Ahmad Salaria</t>
         </is>
       </c>
       <c r="C316" t="n">
@@ -9879,7 +9879,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Muhammad Ilyas Menhas</t>
+          <t>Faisal Mehmood Butt</t>
         </is>
       </c>
       <c r="C317" t="n">
@@ -9921,7 +9921,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Sohaib Manzoor</t>
+          <t>Muhammad Ilyas Menhas</t>
         </is>
       </c>
       <c r="C319" t="n">
@@ -9963,7 +9963,7 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Faisal Mehmood Butt</t>
+          <t>Nouman Ali</t>
         </is>
       </c>
       <c r="C321" t="n">
@@ -9984,7 +9984,7 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Umair Ahmad Salaria</t>
+          <t>Sohaib Manzoor</t>
         </is>
       </c>
       <c r="C322" t="n">
@@ -10005,7 +10005,7 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Tahir Zaidi</t>
+          <t>Wajih H Hashmi</t>
         </is>
       </c>
       <c r="C323" t="n">
@@ -10026,7 +10026,7 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>Rida Javaid</t>
+          <t>Tahir Zaidi</t>
         </is>
       </c>
       <c r="C324" t="n">
@@ -10047,7 +10047,7 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>Wajih H Hashmi</t>
+          <t>Rida Javaid</t>
         </is>
       </c>
       <c r="C325" t="n">
@@ -10068,7 +10068,7 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>Jannat Bakht</t>
+          <t>Qaiser Nadeem</t>
         </is>
       </c>
       <c r="C326" t="n">
@@ -10089,7 +10089,7 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>Qaiser Nadeem</t>
+          <t>Jannat Bakht</t>
         </is>
       </c>
       <c r="C327" t="n">
@@ -10152,7 +10152,7 @@
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>Arslan Usman</t>
+          <t>Daesik Jeong</t>
         </is>
       </c>
       <c r="C330" t="n">
@@ -10173,7 +10173,7 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>Seung Won Lee</t>
+          <t>Hammad Riaz</t>
         </is>
       </c>
       <c r="C331" t="n">
@@ -10194,7 +10194,7 @@
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>Daesik Jeong</t>
+          <t>Seung Won Lee</t>
         </is>
       </c>
       <c r="C332" t="n">
@@ -10215,7 +10215,7 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>Hammad Riaz</t>
+          <t>M Rehan Usman</t>
         </is>
       </c>
       <c r="C333" t="n">
@@ -10236,7 +10236,7 @@
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>M Rehan Usman</t>
+          <t>Arslan Usman</t>
         </is>
       </c>
       <c r="C334" t="n">
@@ -10278,7 +10278,7 @@
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Zixin Guo</t>
+          <t>Wah Hoon Siew</t>
         </is>
       </c>
       <c r="C336" t="n">
@@ -10299,7 +10299,7 @@
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>Guozheng Wang</t>
+          <t>Zixin Guo</t>
         </is>
       </c>
       <c r="C337" t="n">
@@ -10320,7 +10320,7 @@
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>Wah Hoon Siew</t>
+          <t>Guozheng Wang</t>
         </is>
       </c>
       <c r="C338" t="n">
@@ -10362,7 +10362,7 @@
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>Umar Saleem</t>
+          <t>Talha Gul</t>
         </is>
       </c>
       <c r="C340" t="n">
@@ -10404,7 +10404,7 @@
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>Talha Gul</t>
+          <t>Umar Saleem</t>
         </is>
       </c>
       <c r="C342" t="n">
@@ -10425,7 +10425,7 @@
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>Z Ullah</t>
+          <t>Sm Ali</t>
         </is>
       </c>
       <c r="C343" t="n">
@@ -10488,7 +10488,7 @@
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>Sm Ali</t>
+          <t>Z Ullah</t>
         </is>
       </c>
       <c r="C346" t="n">
@@ -10509,7 +10509,7 @@
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>Fuad Usman</t>
+          <t>Ghulam Abbass</t>
         </is>
       </c>
       <c r="C347" t="n">
@@ -10530,7 +10530,7 @@
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>Ghulam Abbass</t>
+          <t>Fuad Usman</t>
         </is>
       </c>
       <c r="C348" t="n">
@@ -10551,7 +10551,7 @@
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>H F Usman</t>
+          <t>S Hamid</t>
         </is>
       </c>
       <c r="C349" t="n">
@@ -10572,7 +10572,7 @@
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>S Hamid</t>
+          <t>H F Usman</t>
         </is>
       </c>
       <c r="C350" t="n">
@@ -10635,7 +10635,7 @@
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>M N Khan</t>
+          <t>W Ali</t>
         </is>
       </c>
       <c r="C353" t="n">
@@ -10656,7 +10656,7 @@
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>W Ali</t>
+          <t>S Kaleem</t>
         </is>
       </c>
       <c r="C354" t="n">
@@ -10677,7 +10677,7 @@
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>S Kaleem</t>
+          <t>M N Khan</t>
         </is>
       </c>
       <c r="C355" t="n">
@@ -10740,7 +10740,7 @@
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>M T Gul</t>
+          <t>M Usman</t>
         </is>
       </c>
       <c r="C358" t="n">
@@ -10761,7 +10761,7 @@
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>M Usman</t>
+          <t>M T Gul</t>
         </is>
       </c>
       <c r="C359" t="n">
@@ -10824,7 +10824,7 @@
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>U Farooq</t>
+          <t>M Nasir</t>
         </is>
       </c>
       <c r="C362" t="n">
@@ -10845,7 +10845,7 @@
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>M Nasir</t>
+          <t>U Farooq</t>
         </is>
       </c>
       <c r="C363" t="n">
@@ -10887,7 +10887,7 @@
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>G B Satrya</t>
+          <t>M R Usman</t>
         </is>
       </c>
       <c r="C365" t="n">
@@ -10908,7 +10908,7 @@
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>M R Usman</t>
+          <t>J Gu</t>
         </is>
       </c>
       <c r="C366" t="n">
@@ -10929,7 +10929,7 @@
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>J Gu</t>
+          <t>G B Satrya</t>
         </is>
       </c>
       <c r="C367" t="n">
@@ -10971,7 +10971,7 @@
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>V Curri</t>
+          <t>A Bianco</t>
         </is>
       </c>
       <c r="C369" t="n">
@@ -11013,7 +11013,7 @@
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>A Bianco</t>
+          <t>V Curri</t>
         </is>
       </c>
       <c r="C371" t="n">
@@ -11076,7 +11076,7 @@
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t>L Potì</t>
+          <t>S Civelli</t>
         </is>
       </c>
       <c r="C374" t="n">
@@ -11118,7 +11118,7 @@
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>N Andriolli</t>
+          <t>M Ferrari</t>
         </is>
       </c>
       <c r="C376" t="n">
@@ -11139,7 +11139,7 @@
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t>A Gatto</t>
+          <t>A Giorgetti</t>
         </is>
       </c>
       <c r="C377" t="n">
@@ -11160,7 +11160,7 @@
       </c>
       <c r="B378" t="inlineStr">
         <is>
-          <t>M Brunero</t>
+          <t>A Gatto</t>
         </is>
       </c>
       <c r="C378" t="n">
@@ -11181,7 +11181,7 @@
       </c>
       <c r="B379" t="inlineStr">
         <is>
-          <t>S Civelli</t>
+          <t>E Paolini</t>
         </is>
       </c>
       <c r="C379" t="n">
@@ -11202,7 +11202,7 @@
       </c>
       <c r="B380" t="inlineStr">
         <is>
-          <t>M Ferrari</t>
+          <t>L Potì</t>
         </is>
       </c>
       <c r="C380" t="n">
@@ -11223,7 +11223,7 @@
       </c>
       <c r="B381" t="inlineStr">
         <is>
-          <t>E Paolini</t>
+          <t>M Brunero</t>
         </is>
       </c>
       <c r="C381" t="n">
@@ -11244,7 +11244,7 @@
       </c>
       <c r="B382" t="inlineStr">
         <is>
-          <t>A Giorgetti</t>
+          <t>N Andriolli</t>
         </is>
       </c>
       <c r="C382" t="n">
@@ -11391,7 +11391,7 @@
       </c>
       <c r="B389" t="inlineStr">
         <is>
-          <t>Shakil Rehman</t>
+          <t>Sheikh</t>
         </is>
       </c>
       <c r="C389" t="n">
@@ -11412,7 +11412,7 @@
       </c>
       <c r="B390" t="inlineStr">
         <is>
-          <t>Sheikh</t>
+          <t>Shakil Rehman</t>
         </is>
       </c>
       <c r="C390" t="n">
@@ -11475,7 +11475,7 @@
       </c>
       <c r="B393" t="inlineStr">
         <is>
-          <t>Ghafoor</t>
+          <t>Nouman</t>
         </is>
       </c>
       <c r="C393" t="n">
@@ -11496,7 +11496,7 @@
       </c>
       <c r="B394" t="inlineStr">
         <is>
-          <t>Nouman</t>
+          <t>Ghafoor</t>
         </is>
       </c>
       <c r="C394" t="n">
@@ -11538,7 +11538,7 @@
       </c>
       <c r="B396" t="inlineStr">
         <is>
-          <t>Bashir Salah</t>
+          <t>Naseer</t>
         </is>
       </c>
       <c r="C396" t="n">
@@ -11559,7 +11559,7 @@
       </c>
       <c r="B397" t="inlineStr">
         <is>
-          <t>Soliman Alkhatib</t>
+          <t>Noman</t>
         </is>
       </c>
       <c r="C397" t="n">
@@ -11580,7 +11580,7 @@
       </c>
       <c r="B398" t="inlineStr">
         <is>
-          <t>Naseer</t>
+          <t>Soliman Alkhatib</t>
         </is>
       </c>
       <c r="C398" t="n">
@@ -11601,7 +11601,7 @@
       </c>
       <c r="B399" t="inlineStr">
         <is>
-          <t>Noman</t>
+          <t>Bashir Salah</t>
         </is>
       </c>
       <c r="C399" t="n">
@@ -11685,7 +11685,7 @@
       </c>
       <c r="B403" t="inlineStr">
         <is>
-          <t>Muhammad</t>
+          <t>Koreshi</t>
         </is>
       </c>
       <c r="C403" t="n">
@@ -11706,7 +11706,7 @@
       </c>
       <c r="B404" t="inlineStr">
         <is>
-          <t>Koreshi</t>
+          <t>Muhammad</t>
         </is>
       </c>
       <c r="C404" t="n">
@@ -11811,7 +11811,7 @@
       </c>
       <c r="B409" t="inlineStr">
         <is>
-          <t>Zia</t>
+          <t>Hafiz Zia Ur Rehman</t>
         </is>
       </c>
       <c r="C409" t="n">
@@ -11832,7 +11832,7 @@
       </c>
       <c r="B410" t="inlineStr">
         <is>
-          <t>Hafiz Zia Ur Rehman</t>
+          <t>Zia</t>
         </is>
       </c>
       <c r="C410" t="n">
@@ -11916,7 +11916,7 @@
       </c>
       <c r="B414" t="inlineStr">
         <is>
-          <t>Ayi Ashyap</t>
+          <t>Ha Majid</t>
         </is>
       </c>
       <c r="C414" t="n">
@@ -11937,7 +11937,7 @@
       </c>
       <c r="B415" t="inlineStr">
         <is>
-          <t>Ha Majid</t>
+          <t>Ayi Ashyap</t>
         </is>
       </c>
       <c r="C415" t="n">
@@ -11958,7 +11958,7 @@
       </c>
       <c r="B416" t="inlineStr">
         <is>
-          <t>Mh Dahri</t>
+          <t>Mi Abbasi</t>
         </is>
       </c>
       <c r="C416" t="n">
@@ -11979,7 +11979,7 @@
       </c>
       <c r="B417" t="inlineStr">
         <is>
-          <t>Mi Abbasi</t>
+          <t>Mh Dahri</t>
         </is>
       </c>
       <c r="C417" t="n">
@@ -12021,7 +12021,7 @@
       </c>
       <c r="B419" t="inlineStr">
         <is>
-          <t>Muhammad Ramlee Kamarudin</t>
+          <t>Yoshihide Yamada</t>
         </is>
       </c>
       <c r="C419" t="n">
@@ -12042,7 +12042,7 @@
       </c>
       <c r="B420" t="inlineStr">
         <is>
-          <t>Zuhairiah Zainal Abidin</t>
+          <t>Nordin Ramli</t>
         </is>
       </c>
       <c r="C420" t="n">
@@ -12063,7 +12063,7 @@
       </c>
       <c r="B421" t="inlineStr">
         <is>
-          <t>Yoshihide Yamada</t>
+          <t>Zuhairiah Zainal Abidin</t>
         </is>
       </c>
       <c r="C421" t="n">
@@ -12084,7 +12084,7 @@
       </c>
       <c r="B422" t="inlineStr">
         <is>
-          <t>Muhammad Hashim Dahri</t>
+          <t>Muhammad Ramlee Kamarudin</t>
         </is>
       </c>
       <c r="C422" t="n">
@@ -12105,7 +12105,7 @@
       </c>
       <c r="B423" t="inlineStr">
         <is>
-          <t>Nordin Ramli</t>
+          <t>Muhammad Hashim Dahri</t>
         </is>
       </c>
       <c r="C423" t="n">
@@ -12126,7 +12126,7 @@
       </c>
       <c r="B424" t="inlineStr">
         <is>
-          <t>Sivathanu Chitra</t>
+          <t>Zuhairiah Z Abidin</t>
         </is>
       </c>
       <c r="C424" t="n">
@@ -12147,7 +12147,7 @@
       </c>
       <c r="B425" t="inlineStr">
         <is>
-          <t>Joseph Charles Vinoth</t>
+          <t>Sivathanu Chitra</t>
         </is>
       </c>
       <c r="C425" t="n">
@@ -12168,7 +12168,7 @@
       </c>
       <c r="B426" t="inlineStr">
         <is>
-          <t>Charles Vinoth</t>
+          <t>Subramaniam Ramesh</t>
         </is>
       </c>
       <c r="C426" t="n">
@@ -12189,7 +12189,7 @@
       </c>
       <c r="B427" t="inlineStr">
         <is>
-          <t>Zuhairiah Z Abidin</t>
+          <t>Charles Vinoth</t>
         </is>
       </c>
       <c r="C427" t="n">
@@ -12210,7 +12210,7 @@
       </c>
       <c r="B428" t="inlineStr">
         <is>
-          <t>Elumalai Saranya</t>
+          <t>Joseph Charles Vinoth</t>
         </is>
       </c>
       <c r="C428" t="n">
@@ -12231,7 +12231,7 @@
       </c>
       <c r="B429" t="inlineStr">
         <is>
-          <t>Subramaniam Ramesh</t>
+          <t>Elumalai Saranya</t>
         </is>
       </c>
       <c r="C429" t="n">
@@ -12483,7 +12483,7 @@
       </c>
       <c r="B441" t="inlineStr">
         <is>
-          <t>D Makri</t>
+          <t>C Mettas</t>
         </is>
       </c>
       <c r="C441" t="n">
@@ -12504,7 +12504,7 @@
       </c>
       <c r="B442" t="inlineStr">
         <is>
-          <t>C Mettas</t>
+          <t>M Tzouvaras</t>
         </is>
       </c>
       <c r="C442" t="n">
@@ -12525,7 +12525,7 @@
       </c>
       <c r="B443" t="inlineStr">
         <is>
-          <t>M Tzouvaras</t>
+          <t>D Makri</t>
         </is>
       </c>
       <c r="C443" t="n">
@@ -12609,7 +12609,7 @@
       </c>
       <c r="B447" t="inlineStr">
         <is>
-          <t>Andrea Buono</t>
+          <t>Samiullah Yousaf</t>
         </is>
       </c>
       <c r="C447" t="n">
@@ -12630,7 +12630,7 @@
       </c>
       <c r="B448" t="inlineStr">
         <is>
-          <t>Maurizio Migliaccio</t>
+          <t>Andrea Buono</t>
         </is>
       </c>
       <c r="C448" t="n">
@@ -12651,7 +12651,7 @@
       </c>
       <c r="B449" t="inlineStr">
         <is>
-          <t>Samiullah Yousaf</t>
+          <t>Maurizio Migliaccio</t>
         </is>
       </c>
       <c r="C449" t="n">
@@ -12714,7 +12714,7 @@
       </c>
       <c r="B452" t="inlineStr">
         <is>
-          <t>Reza Mohammadi</t>
+          <t>Omid Ghozatlou</t>
         </is>
       </c>
       <c r="C452" t="n">
@@ -12735,7 +12735,7 @@
       </c>
       <c r="B453" t="inlineStr">
         <is>
-          <t>Omid Ghozatlou</t>
+          <t>Reza Mohammadi</t>
         </is>
       </c>
       <c r="C453" t="n">
@@ -12798,7 +12798,7 @@
       </c>
       <c r="B456" t="inlineStr">
         <is>
-          <t>Andreas Bathelt</t>
+          <t>Stefan Sieger</t>
         </is>
       </c>
       <c r="C456" t="n">
@@ -12819,7 +12819,7 @@
       </c>
       <c r="B457" t="inlineStr">
         <is>
-          <t>Stefan Sieger</t>
+          <t>Andreas Bathelt</t>
         </is>
       </c>
       <c r="C457" t="n">
@@ -12945,7 +12945,7 @@
       </c>
       <c r="B463" t="inlineStr">
         <is>
-          <t>R Dykstra</t>
+          <t>P Teal</t>
         </is>
       </c>
       <c r="C463" t="n">
@@ -12966,7 +12966,7 @@
       </c>
       <c r="B464" t="inlineStr">
         <is>
-          <t>P Teal</t>
+          <t>R Dykstra</t>
         </is>
       </c>
       <c r="C464" t="n">
@@ -12987,7 +12987,7 @@
       </c>
       <c r="B465" t="inlineStr">
         <is>
-          <t>M Shakeel</t>
+          <t>R Tong</t>
         </is>
       </c>
       <c r="C465" t="n">
@@ -13008,7 +13008,7 @@
       </c>
       <c r="B466" t="inlineStr">
         <is>
-          <t>R Tong</t>
+          <t>M Shakeel</t>
         </is>
       </c>
       <c r="C466" t="n">
@@ -13176,7 +13176,7 @@
       </c>
       <c r="B474" t="inlineStr">
         <is>
-          <t>Imtiaz</t>
+          <t>Asma Talib Qureshi</t>
         </is>
       </c>
       <c r="C474" t="n">
@@ -13197,7 +13197,7 @@
       </c>
       <c r="B475" t="inlineStr">
         <is>
-          <t>Asma Talib Qureshi</t>
+          <t>Imtiaz</t>
         </is>
       </c>
       <c r="C475" t="n">
@@ -13281,7 +13281,7 @@
       </c>
       <c r="B479" t="inlineStr">
         <is>
-          <t>Hassaan Khaliq</t>
+          <t>Waqas Ahmed</t>
         </is>
       </c>
       <c r="C479" t="n">
@@ -13323,7 +13323,7 @@
       </c>
       <c r="B481" t="inlineStr">
         <is>
-          <t>Waqas Ahmed</t>
+          <t>Hassaan Khaliq</t>
         </is>
       </c>
       <c r="C481" t="n">
@@ -13344,7 +13344,7 @@
       </c>
       <c r="B482" t="inlineStr">
         <is>
-          <t>Philippe Bénabès</t>
+          <t>Meseldzija</t>
         </is>
       </c>
       <c r="C482" t="n">
@@ -13365,7 +13365,7 @@
       </c>
       <c r="B483" t="inlineStr">
         <is>
-          <t>Caroline Lelandais Perrault</t>
+          <t>Philippe Bénabès</t>
         </is>
       </c>
       <c r="C483" t="n">
@@ -13386,7 +13386,7 @@
       </c>
       <c r="B484" t="inlineStr">
         <is>
-          <t>Mohamed Ben Chouikha</t>
+          <t>Caroline Lelandais Perrault</t>
         </is>
       </c>
       <c r="C484" t="n">
@@ -13407,7 +13407,7 @@
       </c>
       <c r="B485" t="inlineStr">
         <is>
-          <t>Meseldzija</t>
+          <t>Mohamed Ben Chouikha</t>
         </is>
       </c>
       <c r="C485" t="n">
@@ -13491,7 +13491,7 @@
       </c>
       <c r="B489" t="inlineStr">
         <is>
-          <t>Hamid R Barzegar</t>
+          <t>Nabil El Ioini</t>
         </is>
       </c>
       <c r="C489" t="n">
@@ -13512,7 +13512,7 @@
       </c>
       <c r="B490" t="inlineStr">
         <is>
-          <t>Nabil El Ioini</t>
+          <t>Hamid R Barzegar</t>
         </is>
       </c>
       <c r="C490" t="n">
@@ -13575,7 +13575,7 @@
       </c>
       <c r="B493" t="inlineStr">
         <is>
-          <t>Kashif Hussain</t>
+          <t>Kamil Jalal</t>
         </is>
       </c>
       <c r="C493" t="n">
@@ -13596,7 +13596,7 @@
       </c>
       <c r="B494" t="inlineStr">
         <is>
-          <t>Abdul Wahab</t>
+          <t>Tahir Bashir</t>
         </is>
       </c>
       <c r="C494" t="n">
@@ -13617,7 +13617,7 @@
       </c>
       <c r="B495" t="inlineStr">
         <is>
-          <t>Kamil Jalal</t>
+          <t>Haroon Ahmed</t>
         </is>
       </c>
       <c r="C495" t="n">
@@ -13638,7 +13638,7 @@
       </c>
       <c r="B496" t="inlineStr">
         <is>
-          <t>Tahir Bashir</t>
+          <t>Abdul Wahab</t>
         </is>
       </c>
       <c r="C496" t="n">
@@ -13659,7 +13659,7 @@
       </c>
       <c r="B497" t="inlineStr">
         <is>
-          <t>Haroon Ahmed</t>
+          <t>Kashif Hussain</t>
         </is>
       </c>
       <c r="C497" t="n">
@@ -13701,7 +13701,7 @@
       </c>
       <c r="B499" t="inlineStr">
         <is>
-          <t>Hui Chai</t>
+          <t>Xinhua Wang</t>
         </is>
       </c>
       <c r="C499" t="n">
@@ -13722,7 +13722,7 @@
       </c>
       <c r="B500" t="inlineStr">
         <is>
-          <t>Xinhua Wang</t>
+          <t>Hui Chai</t>
         </is>
       </c>
       <c r="C500" t="n">
@@ -13743,7 +13743,7 @@
       </c>
       <c r="B501" t="inlineStr">
         <is>
-          <t>Yiqi Cheng</t>
+          <t>Farrukh Saleem</t>
         </is>
       </c>
       <c r="C501" t="n">
@@ -13764,7 +13764,7 @@
       </c>
       <c r="B502" t="inlineStr">
         <is>
-          <t>Farrukh Saleem</t>
+          <t>Yiqi Cheng</t>
         </is>
       </c>
       <c r="C502" t="n">
@@ -13785,7 +13785,7 @@
       </c>
       <c r="B503" t="inlineStr">
         <is>
-          <t>He Liu</t>
+          <t>Mingyao Yang</t>
         </is>
       </c>
       <c r="C503" t="n">
@@ -13806,7 +13806,7 @@
       </c>
       <c r="B504" t="inlineStr">
         <is>
-          <t>Zhiyong Huang</t>
+          <t>Pin Wang</t>
         </is>
       </c>
       <c r="C504" t="n">
@@ -13848,7 +13848,7 @@
       </c>
       <c r="B506" t="inlineStr">
         <is>
-          <t>Pin Wang</t>
+          <t>Zhiyong Huang</t>
         </is>
       </c>
       <c r="C506" t="n">
@@ -13890,7 +13890,7 @@
       </c>
       <c r="B508" t="inlineStr">
         <is>
-          <t>Mingyao Yang</t>
+          <t>He Liu</t>
         </is>
       </c>
       <c r="C508" t="n">
@@ -13911,7 +13911,7 @@
       </c>
       <c r="B509" t="inlineStr">
         <is>
-          <t>Fahad R Albogamy</t>
+          <t>Nasim Ullah</t>
         </is>
       </c>
       <c r="C509" t="n">
@@ -13953,7 +13953,7 @@
       </c>
       <c r="B511" t="inlineStr">
         <is>
-          <t>Nasim Ullah</t>
+          <t>Fahad R Albogamy</t>
         </is>
       </c>
       <c r="C511" t="n">
@@ -14016,7 +14016,7 @@
       </c>
       <c r="B514" t="inlineStr">
         <is>
-          <t>Hu Jin</t>
+          <t>Jun Bae Seo</t>
         </is>
       </c>
       <c r="C514" t="n">
@@ -14037,7 +14037,7 @@
       </c>
       <c r="B515" t="inlineStr">
         <is>
-          <t>Jun Bae Seo</t>
+          <t>Hu Jin</t>
         </is>
       </c>
       <c r="C515" t="n">
@@ -14100,7 +14100,7 @@
       </c>
       <c r="B518" t="inlineStr">
         <is>
-          <t>Naeem Maroof</t>
+          <t>Abdul Basit</t>
         </is>
       </c>
       <c r="C518" t="n">
@@ -14121,7 +14121,7 @@
       </c>
       <c r="B519" t="inlineStr">
         <is>
-          <t>Abdul Basit</t>
+          <t>Naeem Maroof</t>
         </is>
       </c>
       <c r="C519" t="n">
@@ -14310,7 +14310,7 @@
       </c>
       <c r="B528" t="inlineStr">
         <is>
-          <t>Muhammad Umair Ahmad Khan</t>
+          <t>Atiqa Saeed</t>
         </is>
       </c>
       <c r="C528" t="n">
@@ -14331,7 +14331,7 @@
       </c>
       <c r="B529" t="inlineStr">
         <is>
-          <t>Hafiz Muhammad Salman Ajmal</t>
+          <t>Muhammad Umair Ahmad Khan</t>
         </is>
       </c>
       <c r="C529" t="n">
@@ -14352,7 +14352,7 @@
       </c>
       <c r="B530" t="inlineStr">
         <is>
-          <t>Atiqa Saeed</t>
+          <t>Hafiz Muhammad Salman Ajmal</t>
         </is>
       </c>
       <c r="C530" t="n">
@@ -14373,7 +14373,7 @@
       </c>
       <c r="B531" t="inlineStr">
         <is>
-          <t>Zaryab Basharat</t>
+          <t>Muhammad Hamza</t>
         </is>
       </c>
       <c r="C531" t="n">
@@ -14394,7 +14394,7 @@
       </c>
       <c r="B532" t="inlineStr">
         <is>
-          <t>Saqlain Abbas</t>
+          <t>Zaryab Basharat</t>
         </is>
       </c>
       <c r="C532" t="n">
@@ -14457,7 +14457,7 @@
       </c>
       <c r="B535" t="inlineStr">
         <is>
-          <t>Muhammad Hamza</t>
+          <t>Saqlain Abbas</t>
         </is>
       </c>
       <c r="C535" t="n">
@@ -14583,7 +14583,7 @@
       </c>
       <c r="B541" t="inlineStr">
         <is>
-          <t>Zohaib Rafi</t>
+          <t>Mujeeb Ur Rehman</t>
         </is>
       </c>
       <c r="C541" t="n">
@@ -14604,7 +14604,7 @@
       </c>
       <c r="B542" t="inlineStr">
         <is>
-          <t>Mujeeb Ur Rehman</t>
+          <t>Muhammad Masab</t>
         </is>
       </c>
       <c r="C542" t="n">
@@ -14625,7 +14625,7 @@
       </c>
       <c r="B543" t="inlineStr">
         <is>
-          <t>Muhammad Masab</t>
+          <t>Zohaib Rafi</t>
         </is>
       </c>
       <c r="C543" t="n">
@@ -14646,7 +14646,7 @@
       </c>
       <c r="B544" t="inlineStr">
         <is>
-          <t>Rabeel Manzoor</t>
+          <t>Farhat Masood</t>
         </is>
       </c>
       <c r="C544" t="n">
@@ -14688,7 +14688,7 @@
       </c>
       <c r="B546" t="inlineStr">
         <is>
-          <t>Farhat Masood</t>
+          <t>Rabeel Manzoor</t>
         </is>
       </c>
       <c r="C546" t="n">
@@ -14751,7 +14751,7 @@
       </c>
       <c r="B549" t="inlineStr">
         <is>
-          <t>Aadil Imran</t>
+          <t>Muhammad Talha Noor</t>
         </is>
       </c>
       <c r="C549" t="n">
@@ -14772,7 +14772,7 @@
       </c>
       <c r="B550" t="inlineStr">
         <is>
-          <t>Shahid Mumtaz</t>
+          <t>Aadil Imran</t>
         </is>
       </c>
       <c r="C550" t="n">
@@ -14793,7 +14793,7 @@
       </c>
       <c r="B551" t="inlineStr">
         <is>
-          <t>Muhammad Talha Noor</t>
+          <t>Shahid Mumtaz</t>
         </is>
       </c>
       <c r="C551" t="n">
@@ -14856,7 +14856,7 @@
       </c>
       <c r="B554" t="inlineStr">
         <is>
-          <t>Dost Muhammad</t>
+          <t>Saqib Bhatti</t>
         </is>
       </c>
       <c r="C554" t="n">
@@ -14877,7 +14877,7 @@
       </c>
       <c r="B555" t="inlineStr">
         <is>
-          <t>Manuel Mazzara</t>
+          <t>Dost Muhammad</t>
         </is>
       </c>
       <c r="C555" t="n">
@@ -14898,7 +14898,7 @@
       </c>
       <c r="B556" t="inlineStr">
         <is>
-          <t>Hafsa Amanullah</t>
+          <t>Manuel Mazzara</t>
         </is>
       </c>
       <c r="C556" t="n">
@@ -14919,7 +14919,7 @@
       </c>
       <c r="B557" t="inlineStr">
         <is>
-          <t>Saqib Bhatti</t>
+          <t>Hafsa Amanullah</t>
         </is>
       </c>
       <c r="C557" t="n">
@@ -14982,7 +14982,7 @@
       </c>
       <c r="B560" t="inlineStr">
         <is>
-          <t>Dick Carrillo Melgarejo</t>
+          <t>Renata Lopes Rosa</t>
         </is>
       </c>
       <c r="C560" t="n">
@@ -15003,7 +15003,7 @@
       </c>
       <c r="B561" t="inlineStr">
         <is>
-          <t>Siti Sarah Maidin</t>
+          <t>Dick Carrillo Melgarejo</t>
         </is>
       </c>
       <c r="C561" t="n">
@@ -15024,7 +15024,7 @@
       </c>
       <c r="B562" t="inlineStr">
         <is>
-          <t>Renata Lopes Rosa</t>
+          <t>Siti Sarah Maidin</t>
         </is>
       </c>
       <c r="C562" t="n">
@@ -15066,7 +15066,7 @@
       </c>
       <c r="B564" t="inlineStr">
         <is>
-          <t>Asif Hussain</t>
+          <t>Hend Khalid Alkahtani</t>
         </is>
       </c>
       <c r="C564" t="n">
@@ -15087,7 +15087,7 @@
       </c>
       <c r="B565" t="inlineStr">
         <is>
-          <t>Zafar Baig</t>
+          <t>Asif Hussain</t>
         </is>
       </c>
       <c r="C565" t="n">
@@ -15108,7 +15108,7 @@
       </c>
       <c r="B566" t="inlineStr">
         <is>
-          <t>Tamara Al Shloul</t>
+          <t>Zafar Baig</t>
         </is>
       </c>
       <c r="C566" t="n">
@@ -15129,7 +15129,7 @@
       </c>
       <c r="B567" t="inlineStr">
         <is>
-          <t>Hend Khalid Alkahtani</t>
+          <t>Tamara Al Shloul</t>
         </is>
       </c>
       <c r="C567" t="n">
@@ -15150,7 +15150,7 @@
       </c>
       <c r="B568" t="inlineStr">
         <is>
-          <t>Muhammad Adnan</t>
+          <t>Fuad A Awwad</t>
         </is>
       </c>
       <c r="C568" t="n">
@@ -15171,7 +15171,7 @@
       </c>
       <c r="B569" t="inlineStr">
         <is>
-          <t>Syed Rehan Ashraf</t>
+          <t>Mohamed R Abonazel</t>
         </is>
       </c>
       <c r="C569" t="n">
@@ -15192,7 +15192,7 @@
       </c>
       <c r="B570" t="inlineStr">
         <is>
-          <t>Muhammad Hybrid</t>
+          <t>Muhammad Asim Butt</t>
         </is>
       </c>
       <c r="C570" t="n">
@@ -15213,7 +15213,7 @@
       </c>
       <c r="B571" t="inlineStr">
         <is>
-          <t>Izaz Hassan</t>
+          <t>Khalid Ijaz</t>
         </is>
       </c>
       <c r="C571" t="n">
@@ -15234,7 +15234,7 @@
       </c>
       <c r="B572" t="inlineStr">
         <is>
-          <t>Fuad A Awwad</t>
+          <t>Muhammad Hybrid</t>
         </is>
       </c>
       <c r="C572" t="n">
@@ -15255,7 +15255,7 @@
       </c>
       <c r="B573" t="inlineStr">
         <is>
-          <t>Khalid Ijaz</t>
+          <t>Syed Rehan Ashraf</t>
         </is>
       </c>
       <c r="C573" t="n">
@@ -15276,7 +15276,7 @@
       </c>
       <c r="B574" t="inlineStr">
         <is>
-          <t>Mohamed R Abonazel</t>
+          <t>Muhammad Adnan</t>
         </is>
       </c>
       <c r="C574" t="n">
@@ -15297,7 +15297,7 @@
       </c>
       <c r="B575" t="inlineStr">
         <is>
-          <t>Muhammad Asim Butt</t>
+          <t>Izaz Hassan</t>
         </is>
       </c>
       <c r="C575" t="n">
@@ -15318,7 +15318,7 @@
       </c>
       <c r="B576" t="inlineStr">
         <is>
-          <t>Junaid Imtiaz</t>
+          <t>Amira Syed A Aziz</t>
         </is>
       </c>
       <c r="C576" t="n">
@@ -15339,7 +15339,7 @@
       </c>
       <c r="B577" t="inlineStr">
         <is>
-          <t>El Awadi Attia</t>
+          <t>Muhammad Assam</t>
         </is>
       </c>
       <c r="C577" t="n">
@@ -15360,7 +15360,7 @@
       </c>
       <c r="B578" t="inlineStr">
         <is>
-          <t>Amira Syed A Aziz</t>
+          <t>El Awadi Attia</t>
         </is>
       </c>
       <c r="C578" t="n">
@@ -15381,7 +15381,7 @@
       </c>
       <c r="B579" t="inlineStr">
         <is>
-          <t>Muhammad Assam</t>
+          <t>Junaid Imtiaz</t>
         </is>
       </c>
       <c r="C579" t="n">
@@ -15423,7 +15423,7 @@
       </c>
       <c r="B581" t="inlineStr">
         <is>
-          <t>Saddique Khalid</t>
+          <t>Muhammad Shoaib</t>
         </is>
       </c>
       <c r="C581" t="n">
@@ -15465,7 +15465,7 @@
       </c>
       <c r="B583" t="inlineStr">
         <is>
-          <t>Muhammad Shoaib</t>
+          <t>Saddique Khalid</t>
         </is>
       </c>
       <c r="C583" t="n">
@@ -15486,7 +15486,7 @@
       </c>
       <c r="B584" t="inlineStr">
         <is>
-          <t>Umair Bajwa</t>
+          <t>Anees Ur Rehman</t>
         </is>
       </c>
       <c r="C584" t="n">
@@ -15528,7 +15528,7 @@
       </c>
       <c r="B586" t="inlineStr">
         <is>
-          <t>Anees Ur Rehman</t>
+          <t>Umair Bajwa</t>
         </is>
       </c>
       <c r="C586" t="n">
@@ -15633,7 +15633,7 @@
       </c>
       <c r="B591" t="inlineStr">
         <is>
-          <t>Farah Khalid</t>
+          <t>Muhammad Farhan</t>
         </is>
       </c>
       <c r="C591" t="n">
@@ -15654,7 +15654,7 @@
       </c>
       <c r="B592" t="inlineStr">
         <is>
-          <t>Muhammad Farhan</t>
+          <t>Farah Khalid</t>
         </is>
       </c>
       <c r="C592" t="n">
@@ -15843,7 +15843,7 @@
       </c>
       <c r="B601" t="inlineStr">
         <is>
-          <t>Huseyin Arslan</t>
+          <t>Mehmet Ali Aygul</t>
         </is>
       </c>
       <c r="C601" t="n">
@@ -15864,7 +15864,7 @@
       </c>
       <c r="B602" t="inlineStr">
         <is>
-          <t>Mehmet Ali Aygul</t>
+          <t>Huseyin Arslan</t>
         </is>
       </c>
       <c r="C602" t="n">
@@ -16116,7 +16116,7 @@
       </c>
       <c r="B614" t="inlineStr">
         <is>
-          <t>Ashfaq Ahmed</t>
+          <t>Adnan Zafar</t>
         </is>
       </c>
       <c r="C614" t="n">
@@ -16137,7 +16137,7 @@
       </c>
       <c r="B615" t="inlineStr">
         <is>
-          <t>Adnan Zafar</t>
+          <t>Ashfaq Ahmed</t>
         </is>
       </c>
       <c r="C615" t="n">
@@ -16158,7 +16158,7 @@
       </c>
       <c r="B616" t="inlineStr">
         <is>
-          <t>Qureshi</t>
+          <t>Hassaan Khaliq</t>
         </is>
       </c>
       <c r="C616" t="n">
@@ -16179,7 +16179,7 @@
       </c>
       <c r="B617" t="inlineStr">
         <is>
-          <t>Hassaan Khaliq</t>
+          <t>Qureshi</t>
         </is>
       </c>
       <c r="C617" t="n">
@@ -16326,7 +16326,7 @@
       </c>
       <c r="B624" t="inlineStr">
         <is>
-          <t>Chang Qing Dong</t>
+          <t>Zafar Hussain</t>
         </is>
       </c>
       <c r="C624" t="n">
@@ -16347,7 +16347,7 @@
       </c>
       <c r="B625" t="inlineStr">
         <is>
-          <t>Qiang Lu</t>
+          <t>Adnan Abbas</t>
         </is>
       </c>
       <c r="C625" t="n">
@@ -16368,7 +16368,7 @@
       </c>
       <c r="B626" t="inlineStr">
         <is>
-          <t>Zulfiqar Ali</t>
+          <t>Chang Qing Dong</t>
         </is>
       </c>
       <c r="C626" t="n">
@@ -16389,7 +16389,7 @@
       </c>
       <c r="B627" t="inlineStr">
         <is>
-          <t>Zafar Hussain</t>
+          <t>Qiang Lu</t>
         </is>
       </c>
       <c r="C627" t="n">
@@ -16410,7 +16410,7 @@
       </c>
       <c r="B628" t="inlineStr">
         <is>
-          <t>Adnan Abbas</t>
+          <t>Zulfiqar Ali</t>
         </is>
       </c>
       <c r="C628" t="n">
@@ -16515,7 +16515,7 @@
       </c>
       <c r="B633" t="inlineStr">
         <is>
-          <t>Mohan Menghwar</t>
+          <t>Li Meicheng</t>
         </is>
       </c>
       <c r="C633" t="n">
@@ -16536,7 +16536,7 @@
       </c>
       <c r="B634" t="inlineStr">
         <is>
-          <t>Li Meicheng</t>
+          <t>Mohan Menghwar</t>
         </is>
       </c>
       <c r="C634" t="n">
@@ -16557,7 +16557,7 @@
       </c>
       <c r="B635" t="inlineStr">
         <is>
-          <t>Zulqarnain Arain</t>
+          <t>Min Xing Zhou</t>
         </is>
       </c>
       <c r="C635" t="n">
@@ -16578,7 +16578,7 @@
       </c>
       <c r="B636" t="inlineStr">
         <is>
-          <t>Min Xing Zhou</t>
+          <t>Zulqarnain Arain</t>
         </is>
       </c>
       <c r="C636" t="n">
@@ -16620,7 +16620,7 @@
       </c>
       <c r="B638" t="inlineStr">
         <is>
-          <t>Chengrong Li</t>
+          <t>Yuzhen Lv</t>
         </is>
       </c>
       <c r="C638" t="n">
@@ -16641,7 +16641,7 @@
       </c>
       <c r="B639" t="inlineStr">
         <is>
-          <t>Yuzhen Lv</t>
+          <t>Chengrong Li</t>
         </is>
       </c>
       <c r="C639" t="n">
@@ -16662,7 +16662,7 @@
       </c>
       <c r="B640" t="inlineStr">
         <is>
-          <t>Hu Zhifeng</t>
+          <t>Kai Yi</t>
         </is>
       </c>
       <c r="C640" t="n">
@@ -16683,7 +16683,7 @@
       </c>
       <c r="B641" t="inlineStr">
         <is>
-          <t>Kai Yi</t>
+          <t>Hu Zhifeng</t>
         </is>
       </c>
       <c r="C641" t="n">
@@ -16704,7 +16704,7 @@
       </c>
       <c r="B642" t="inlineStr">
         <is>
-          <t>Farukh Abbas</t>
+          <t>Syed Furqan Rafique</t>
         </is>
       </c>
       <c r="C642" t="n">
@@ -16725,7 +16725,7 @@
       </c>
       <c r="B643" t="inlineStr">
         <is>
-          <t>Syed Furqan Rafique</t>
+          <t>Farukh Abbas</t>
         </is>
       </c>
       <c r="C643" t="n">
@@ -16746,7 +16746,7 @@
       </c>
       <c r="B644" t="inlineStr">
         <is>
-          <t>Hasan Ul Banna</t>
+          <t>Arsham Iqbal</t>
         </is>
       </c>
       <c r="C644" t="n">
@@ -16767,7 +16767,7 @@
       </c>
       <c r="B645" t="inlineStr">
         <is>
-          <t>Ibrahim F</t>
+          <t>Hasan Ul Banna</t>
         </is>
       </c>
       <c r="C645" t="n">
@@ -16809,7 +16809,7 @@
       </c>
       <c r="B647" t="inlineStr">
         <is>
-          <t>Arsham Iqbal</t>
+          <t>Ibrahim F</t>
         </is>
       </c>
       <c r="C647" t="n">
@@ -16872,7 +16872,7 @@
       </c>
       <c r="B650" t="inlineStr">
         <is>
-          <t>Akhtar Hussain</t>
+          <t>Nauman Ahmad Zaffar</t>
         </is>
       </c>
       <c r="C650" t="n">
@@ -16914,7 +16914,7 @@
       </c>
       <c r="B652" t="inlineStr">
         <is>
-          <t>Nauman Ahmad Zaffar</t>
+          <t>Akhtar Hussain</t>
         </is>
       </c>
       <c r="C652" t="n">
@@ -16998,7 +16998,7 @@
       </c>
       <c r="B656" t="inlineStr">
         <is>
-          <t>Sugiyama</t>
+          <t>Nakano</t>
         </is>
       </c>
       <c r="C656" t="n">
@@ -17040,7 +17040,7 @@
       </c>
       <c r="B658" t="inlineStr">
         <is>
-          <t>Fujii</t>
+          <t>Sugiyama</t>
         </is>
       </c>
       <c r="C658" t="n">
@@ -17082,7 +17082,7 @@
       </c>
       <c r="B660" t="inlineStr">
         <is>
-          <t>Nakano</t>
+          <t>Fujii</t>
         </is>
       </c>
       <c r="C660" t="n">
@@ -17166,7 +17166,7 @@
       </c>
       <c r="B664" t="inlineStr">
         <is>
-          <t>R Abdul Karim</t>
+          <t>M R</t>
         </is>
       </c>
       <c r="C664" t="n">
@@ -17187,7 +17187,7 @@
       </c>
       <c r="B665" t="inlineStr">
         <is>
-          <t>M R</t>
+          <t>R Abdul Karim</t>
         </is>
       </c>
       <c r="C665" t="n">
@@ -17208,7 +17208,7 @@
       </c>
       <c r="B666" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>Karim</t>
         </is>
       </c>
       <c r="C666" t="n">
@@ -17229,7 +17229,7 @@
       </c>
       <c r="B667" t="inlineStr">
         <is>
-          <t>M R A</t>
+          <t>M A</t>
         </is>
       </c>
       <c r="C667" t="n">
@@ -17250,7 +17250,7 @@
       </c>
       <c r="B668" t="inlineStr">
         <is>
-          <t>Marwat</t>
+          <t>M R A</t>
         </is>
       </c>
       <c r="C668" t="n">
@@ -17271,7 +17271,7 @@
       </c>
       <c r="B669" t="inlineStr">
         <is>
-          <t>M A</t>
+          <t>R</t>
         </is>
       </c>
       <c r="C669" t="n">
@@ -17292,7 +17292,7 @@
       </c>
       <c r="B670" t="inlineStr">
         <is>
-          <t>Karim</t>
+          <t>Marwat</t>
         </is>
       </c>
       <c r="C670" t="n">
@@ -17313,7 +17313,7 @@
       </c>
       <c r="B671" t="inlineStr">
         <is>
-          <t>T H</t>
+          <t>Haider</t>
         </is>
       </c>
       <c r="C671" t="n">
@@ -17334,7 +17334,7 @@
       </c>
       <c r="B672" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>T H</t>
         </is>
       </c>
       <c r="C672" t="n">
@@ -17355,7 +17355,7 @@
       </c>
       <c r="B673" t="inlineStr">
         <is>
-          <t>Nadeem</t>
+          <t>S</t>
         </is>
       </c>
       <c r="C673" t="n">
@@ -17376,7 +17376,7 @@
       </c>
       <c r="B674" t="inlineStr">
         <is>
-          <t>M M</t>
+          <t>Daas</t>
         </is>
       </c>
       <c r="C674" t="n">
@@ -17397,7 +17397,7 @@
       </c>
       <c r="B675" t="inlineStr">
         <is>
-          <t>Haider</t>
+          <t>M M</t>
         </is>
       </c>
       <c r="C675" t="n">
@@ -17418,7 +17418,7 @@
       </c>
       <c r="B676" t="inlineStr">
         <is>
-          <t>Daas</t>
+          <t>Nadeem</t>
         </is>
       </c>
       <c r="C676" t="n">
@@ -17481,7 +17481,7 @@
       </c>
       <c r="B679" t="inlineStr">
         <is>
-          <t>A A</t>
+          <t>Kolesnikov</t>
         </is>
       </c>
       <c r="C679" t="n">
@@ -17502,7 +17502,7 @@
       </c>
       <c r="B680" t="inlineStr">
         <is>
-          <t>Y S</t>
+          <t>A A</t>
         </is>
       </c>
       <c r="C680" t="n">
@@ -17523,7 +17523,7 @@
       </c>
       <c r="B681" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Kurochkin</t>
         </is>
       </c>
       <c r="C681" t="n">
@@ -17544,7 +17544,7 @@
       </c>
       <c r="B682" t="inlineStr">
         <is>
-          <t>Razumtecev</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C682" t="n">
@@ -17565,7 +17565,7 @@
       </c>
       <c r="B683" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>Y S</t>
         </is>
       </c>
       <c r="C683" t="n">
@@ -17586,7 +17586,7 @@
       </c>
       <c r="B684" t="inlineStr">
         <is>
-          <t>Kolesnikov</t>
+          <t>I</t>
         </is>
       </c>
       <c r="C684" t="n">
@@ -17607,7 +17607,7 @@
       </c>
       <c r="B685" t="inlineStr">
         <is>
-          <t>Kurochkin</t>
+          <t>Razumtecev</t>
         </is>
       </c>
       <c r="C685" t="n">
@@ -17628,7 +17628,7 @@
       </c>
       <c r="B686" t="inlineStr">
         <is>
-          <t>Walaa Alayed</t>
+          <t>Momna Ikram</t>
         </is>
       </c>
       <c r="C686" t="n">
@@ -17649,7 +17649,7 @@
       </c>
       <c r="B687" t="inlineStr">
         <is>
-          <t>Momna Ikram</t>
+          <t>Walaa Alayed</t>
         </is>
       </c>
       <c r="C687" t="n">
@@ -17670,7 +17670,7 @@
       </c>
       <c r="B688" t="inlineStr">
         <is>
-          <t>Ahmed Zeeshan</t>
+          <t>Dilawar Hussain</t>
         </is>
       </c>
       <c r="C688" t="n">
@@ -17691,7 +17691,7 @@
       </c>
       <c r="B689" t="inlineStr">
         <is>
-          <t>Zaheer Asghar</t>
+          <t>Ahmed Zeeshan</t>
         </is>
       </c>
       <c r="C689" t="n">
@@ -17712,7 +17712,7 @@
       </c>
       <c r="B690" t="inlineStr">
         <is>
-          <t>Dilawar Hussain</t>
+          <t>Zaheer Asghar</t>
         </is>
       </c>
       <c r="C690" t="n">
@@ -17733,7 +17733,7 @@
       </c>
       <c r="B691" t="inlineStr">
         <is>
-          <t>Youssef N Altherwy</t>
+          <t>Syed Rameez Naqvi</t>
         </is>
       </c>
       <c r="C691" t="n">
@@ -17754,7 +17754,7 @@
       </c>
       <c r="B692" t="inlineStr">
         <is>
-          <t>Syed Rameez Naqvi</t>
+          <t>Tallha Akram</t>
         </is>
       </c>
       <c r="C692" t="n">
@@ -17775,7 +17775,7 @@
       </c>
       <c r="B693" t="inlineStr">
         <is>
-          <t>Bilal Ahmed</t>
+          <t>Youssef N Altherwy</t>
         </is>
       </c>
       <c r="C693" t="n">
@@ -17796,7 +17796,7 @@
       </c>
       <c r="B694" t="inlineStr">
         <is>
-          <t>Tallha Akram</t>
+          <t>Bilal Ahmed</t>
         </is>
       </c>
       <c r="C694" t="n">
@@ -17838,7 +17838,7 @@
       </c>
       <c r="B696" t="inlineStr">
         <is>
-          <t>Qaiser Hussain</t>
+          <t>Gulistan Raja</t>
         </is>
       </c>
       <c r="C696" t="n">
@@ -17859,7 +17859,7 @@
       </c>
       <c r="B697" t="inlineStr">
         <is>
-          <t>Gulistan Raja</t>
+          <t>Qaiser Hussain</t>
         </is>
       </c>
       <c r="C697" t="n">
@@ -18006,7 +18006,7 @@
       </c>
       <c r="B704" t="inlineStr">
         <is>
-          <t>Syed Ali Raza Zaidi</t>
+          <t>Rafia Mumtaz</t>
         </is>
       </c>
       <c r="C704" t="n">
@@ -18027,7 +18027,7 @@
       </c>
       <c r="B705" t="inlineStr">
         <is>
-          <t>Rafia Mumtaz</t>
+          <t>Syed Ali Raza Zaidi</t>
         </is>
       </c>
       <c r="C705" t="n">
@@ -18111,7 +18111,7 @@
       </c>
       <c r="B709" t="inlineStr">
         <is>
-          <t>Hassaan Khaliq</t>
+          <t>Kapal Dev</t>
         </is>
       </c>
       <c r="C709" t="n">
@@ -18132,7 +18132,7 @@
       </c>
       <c r="B710" t="inlineStr">
         <is>
-          <t>Kapal Dev</t>
+          <t>Hassaan Khaliq</t>
         </is>
       </c>
       <c r="C710" t="n">
@@ -18216,7 +18216,7 @@
       </c>
       <c r="B714" t="inlineStr">
         <is>
-          <t>Rashid Ali</t>
+          <t>Amir Haider</t>
         </is>
       </c>
       <c r="C714" t="n">
@@ -18237,7 +18237,7 @@
       </c>
       <c r="B715" t="inlineStr">
         <is>
-          <t>Amir Haider</t>
+          <t>Rashid Ali</t>
         </is>
       </c>
       <c r="C715" t="n">
@@ -18279,7 +18279,7 @@
       </c>
       <c r="B717" t="inlineStr">
         <is>
-          <t>J Chung</t>
+          <t>R Kettimuthu</t>
         </is>
       </c>
       <c r="C717" t="n">
@@ -18300,7 +18300,7 @@
       </c>
       <c r="B718" t="inlineStr">
         <is>
-          <t>R Kettimuthu</t>
+          <t>J Chung</t>
         </is>
       </c>
       <c r="C718" t="n">
@@ -18405,7 +18405,7 @@
       </c>
       <c r="B723" t="inlineStr">
         <is>
-          <t>Umais Khan</t>
+          <t>Sarim Farqaleet Khan</t>
         </is>
       </c>
       <c r="C723" t="n">
@@ -18426,7 +18426,7 @@
       </c>
       <c r="B724" t="inlineStr">
         <is>
-          <t>Sarim Farqaleet Khan</t>
+          <t>Umais Khan</t>
         </is>
       </c>
       <c r="C724" t="n">
@@ -18468,7 +18468,7 @@
       </c>
       <c r="B726" t="inlineStr">
         <is>
-          <t>Iu Khalil</t>
+          <t>Abraiz Khattak</t>
         </is>
       </c>
       <c r="C726" t="n">
@@ -18489,7 +18489,7 @@
       </c>
       <c r="B727" t="inlineStr">
         <is>
-          <t>Abraiz Khattak</t>
+          <t>Iu Khalil</t>
         </is>
       </c>
       <c r="C727" t="n">
@@ -18678,7 +18678,7 @@
       </c>
       <c r="B736" t="inlineStr">
         <is>
-          <t>Qudratullah Wazir</t>
+          <t>Saifullah Khan</t>
         </is>
       </c>
       <c r="C736" t="n">
@@ -18699,7 +18699,7 @@
       </c>
       <c r="B737" t="inlineStr">
         <is>
-          <t>Saifullah Khan</t>
+          <t>Faiza Hayat</t>
         </is>
       </c>
       <c r="C737" t="n">
@@ -18720,7 +18720,7 @@
       </c>
       <c r="B738" t="inlineStr">
         <is>
-          <t>Faiza Hayat</t>
+          <t>Qudratullah Wazir</t>
         </is>
       </c>
       <c r="C738" t="n">
@@ -19329,7 +19329,7 @@
       </c>
       <c r="B767" t="inlineStr">
         <is>
-          <t>Abdul Shakoor</t>
+          <t>Sikander Azam</t>
         </is>
       </c>
       <c r="C767" t="n">
@@ -19350,7 +19350,7 @@
       </c>
       <c r="B768" t="inlineStr">
         <is>
-          <t>Fakhra Ghafoor</t>
+          <t>H W Seo</t>
         </is>
       </c>
       <c r="C768" t="n">
@@ -19371,7 +19371,7 @@
       </c>
       <c r="B769" t="inlineStr">
         <is>
-          <t>Bakhtiar Ul Haq</t>
+          <t>Abdul Shakoor</t>
         </is>
       </c>
       <c r="C769" t="n">
@@ -19392,7 +19392,7 @@
       </c>
       <c r="B770" t="inlineStr">
         <is>
-          <t>H W Seo</t>
+          <t>Fakhra Ghafoor</t>
         </is>
       </c>
       <c r="C770" t="n">
@@ -19434,7 +19434,7 @@
       </c>
       <c r="B772" t="inlineStr">
         <is>
-          <t>Sikander Azam</t>
+          <t>Bakhtiar Ul Haq</t>
         </is>
       </c>
       <c r="C772" t="n">
@@ -19455,7 +19455,7 @@
       </c>
       <c r="B773" t="inlineStr">
         <is>
-          <t>Zahir Abbas</t>
+          <t>Syed Adil Sardar</t>
         </is>
       </c>
       <c r="C773" t="n">
@@ -19476,7 +19476,7 @@
       </c>
       <c r="B774" t="inlineStr">
         <is>
-          <t>Syed Adil Sardar</t>
+          <t>Zahir Abbas</t>
         </is>
       </c>
       <c r="C774" t="n">
@@ -19539,7 +19539,7 @@
       </c>
       <c r="B777" t="inlineStr">
         <is>
-          <t>Jahan Zeb Gul</t>
+          <t>Rui Chang</t>
         </is>
       </c>
       <c r="C777" t="n">
@@ -19560,7 +19560,7 @@
       </c>
       <c r="B778" t="inlineStr">
         <is>
-          <t>Rayyan Ali Shaukat</t>
+          <t>Jahan Zeb Gul</t>
         </is>
       </c>
       <c r="C778" t="n">
@@ -19581,7 +19581,7 @@
       </c>
       <c r="B779" t="inlineStr">
         <is>
-          <t>Yarjan Abdul Samad</t>
+          <t>Yijun Shi</t>
         </is>
       </c>
       <c r="C779" t="n">
@@ -19602,7 +19602,7 @@
       </c>
       <c r="B780" t="inlineStr">
         <is>
-          <t>Yijun Shi</t>
+          <t>Rayyan Ali Shaukat</t>
         </is>
       </c>
       <c r="C780" t="n">
@@ -19623,7 +19623,7 @@
       </c>
       <c r="B781" t="inlineStr">
         <is>
-          <t>Rui Chang</t>
+          <t>Yarjan Abdul Samad</t>
         </is>
       </c>
       <c r="C781" t="n">
@@ -19644,7 +19644,7 @@
       </c>
       <c r="B782" t="inlineStr">
         <is>
-          <t>Ghayas Uddin Siddiqui</t>
+          <t>Ahmed Usman Ali</t>
         </is>
       </c>
       <c r="C782" t="n">
@@ -19665,7 +19665,7 @@
       </c>
       <c r="B783" t="inlineStr">
         <is>
-          <t>Ahmed Usman Ali</t>
+          <t>Ghayas Uddin Siddiqui</t>
         </is>
       </c>
       <c r="C783" t="n">
@@ -19749,7 +19749,7 @@
       </c>
       <c r="B787" t="inlineStr">
         <is>
-          <t>Bernabe Mari</t>
+          <t>Yousaf Hameed Khattak</t>
         </is>
       </c>
       <c r="C787" t="n">
@@ -19770,7 +19770,7 @@
       </c>
       <c r="B788" t="inlineStr">
         <is>
-          <t>Faisal Baig</t>
+          <t>Bernabe Mari</t>
         </is>
       </c>
       <c r="C788" t="n">
@@ -19791,7 +19791,7 @@
       </c>
       <c r="B789" t="inlineStr">
         <is>
-          <t>Anzar Mahmood</t>
+          <t>Faisal Baig</t>
         </is>
       </c>
       <c r="C789" t="n">
@@ -19812,7 +19812,7 @@
       </c>
       <c r="B790" t="inlineStr">
         <is>
-          <t>Yousaf Hameed Khattak</t>
+          <t>Anzar Mahmood</t>
         </is>
       </c>
       <c r="C790" t="n">
@@ -20085,7 +20085,7 @@
       </c>
       <c r="B803" t="inlineStr">
         <is>
-          <t>Faheem Khuhawar</t>
+          <t>Muhammad Talha Amin</t>
         </is>
       </c>
       <c r="C803" t="n">
@@ -20106,7 +20106,7 @@
       </c>
       <c r="B804" t="inlineStr">
         <is>
-          <t>Muhammad Talha Amin</t>
+          <t>Hafsa Shaikh</t>
         </is>
       </c>
       <c r="C804" t="n">
@@ -20127,7 +20127,7 @@
       </c>
       <c r="B805" t="inlineStr">
         <is>
-          <t>Hafsa Shaikh</t>
+          <t>Faheem Khuhawar</t>
         </is>
       </c>
       <c r="C805" t="n">
@@ -20148,7 +20148,7 @@
       </c>
       <c r="B806" t="inlineStr">
         <is>
-          <t>Tehmina Kalsum</t>
+          <t>Hafiz Arslan Ramzan</t>
         </is>
       </c>
       <c r="C806" t="n">
@@ -20169,7 +20169,7 @@
       </c>
       <c r="B807" t="inlineStr">
         <is>
-          <t>Sadia Ramzan</t>
+          <t>Tehmina Kalsum</t>
         </is>
       </c>
       <c r="C807" t="n">
@@ -20190,7 +20190,7 @@
       </c>
       <c r="B808" t="inlineStr">
         <is>
-          <t>Hafiz Arslan Ramzan</t>
+          <t>Sadia Ramzan</t>
         </is>
       </c>
       <c r="C808" t="n">
@@ -20337,7 +20337,7 @@
       </c>
       <c r="B815" t="inlineStr">
         <is>
-          <t>Furqan Rustam</t>
+          <t>Hafeez Ur Rehman</t>
         </is>
       </c>
       <c r="C815" t="n">
@@ -20358,7 +20358,7 @@
       </c>
       <c r="B816" t="inlineStr">
         <is>
-          <t>Hafeez Ur Rehman</t>
+          <t>Furqan Rustam</t>
         </is>
       </c>
       <c r="C816" t="n">
@@ -20526,7 +20526,7 @@
       </c>
       <c r="B824" t="inlineStr">
         <is>
-          <t>Divya Velayudhan</t>
+          <t>Samet Akcay</t>
         </is>
       </c>
       <c r="C824" t="n">
@@ -20568,7 +20568,7 @@
       </c>
       <c r="B826" t="inlineStr">
         <is>
-          <t>Samet Akcay</t>
+          <t>Divya Velayudhan</t>
         </is>
       </c>
       <c r="C826" t="n">
@@ -20589,7 +20589,7 @@
       </c>
       <c r="B827" t="inlineStr">
         <is>
-          <t>Muhammad Shahzad</t>
+          <t>Aisha Gul Hafeez</t>
         </is>
       </c>
       <c r="C827" t="n">
@@ -20610,7 +20610,7 @@
       </c>
       <c r="B828" t="inlineStr">
         <is>
-          <t>Aisha Gul Hafeez</t>
+          <t>Muhammad Shahzad</t>
         </is>
       </c>
       <c r="C828" t="n">
@@ -20715,7 +20715,7 @@
       </c>
       <c r="B833" t="inlineStr">
         <is>
-          <t>Farrukh Javed Gill</t>
+          <t>Imran Farid Nizami</t>
         </is>
       </c>
       <c r="C833" t="n">
@@ -20736,7 +20736,7 @@
       </c>
       <c r="B834" t="inlineStr">
         <is>
-          <t>Mobeen Ur Rahman</t>
+          <t>Farrukh Javed Gill</t>
         </is>
       </c>
       <c r="C834" t="n">
@@ -20757,7 +20757,7 @@
       </c>
       <c r="B835" t="inlineStr">
         <is>
-          <t>Imran Farid Nizami</t>
+          <t>Mobeen Ur Rahman</t>
         </is>
       </c>
       <c r="C835" t="n">
@@ -20862,7 +20862,7 @@
       </c>
       <c r="B840" t="inlineStr">
         <is>
-          <t>Hassan Kazmi</t>
+          <t>Aitzaz Saleem</t>
         </is>
       </c>
       <c r="C840" t="n">
@@ -20883,7 +20883,7 @@
       </c>
       <c r="B841" t="inlineStr">
         <is>
-          <t>Aitzaz Saleem</t>
+          <t>Hassan Kazmi</t>
         </is>
       </c>
       <c r="C841" t="n">
@@ -21009,7 +21009,7 @@
       </c>
       <c r="B847" t="inlineStr">
         <is>
-          <t>Soyiba Jawed</t>
+          <t>Jahan Zeb</t>
         </is>
       </c>
       <c r="C847" t="n">
@@ -21030,7 +21030,7 @@
       </c>
       <c r="B848" t="inlineStr">
         <is>
-          <t>Jahan Zeb</t>
+          <t>Soyiba Jawed</t>
         </is>
       </c>
       <c r="C848" t="n">
@@ -21093,7 +21093,7 @@
       </c>
       <c r="B851" t="inlineStr">
         <is>
-          <t>Amina Jameel</t>
+          <t>Samina Khalid</t>
         </is>
       </c>
       <c r="C851" t="n">
@@ -21114,7 +21114,7 @@
       </c>
       <c r="B852" t="inlineStr">
         <is>
-          <t>Samina Khalid</t>
+          <t>Amina Jameel</t>
         </is>
       </c>
       <c r="C852" t="n">
@@ -21135,7 +21135,7 @@
       </c>
       <c r="B853" t="inlineStr">
         <is>
-          <t>Khawar Khurshid</t>
+          <t>Imran Fareed Nizami</t>
         </is>
       </c>
       <c r="C853" t="n">
@@ -21156,7 +21156,7 @@
       </c>
       <c r="B854" t="inlineStr">
         <is>
-          <t>Imran Fareed Nizami</t>
+          <t>Muhammad Majid</t>
         </is>
       </c>
       <c r="C854" t="n">
@@ -21177,7 +21177,7 @@
       </c>
       <c r="B855" t="inlineStr">
         <is>
-          <t>Mobeen Ur Rehman</t>
+          <t>Syed Muhammad Anwar</t>
         </is>
       </c>
       <c r="C855" t="n">
@@ -21198,7 +21198,7 @@
       </c>
       <c r="B856" t="inlineStr">
         <is>
-          <t>Syed Muhammad Anwar</t>
+          <t>Mobeen Ur Rehman</t>
         </is>
       </c>
       <c r="C856" t="n">
@@ -21219,7 +21219,7 @@
       </c>
       <c r="B857" t="inlineStr">
         <is>
-          <t>Muhammad Majid</t>
+          <t>Khawar Khurshid</t>
         </is>
       </c>
       <c r="C857" t="n">
@@ -21240,7 +21240,7 @@
       </c>
       <c r="B858" t="inlineStr">
         <is>
-          <t>Arslan Shaukat</t>
+          <t>Anum Abdus Salam</t>
         </is>
       </c>
       <c r="C858" t="n">
@@ -21261,7 +21261,7 @@
       </c>
       <c r="B859" t="inlineStr">
         <is>
-          <t>Anum Abdus Salam</t>
+          <t>And Muhammad Usman Akram</t>
         </is>
       </c>
       <c r="C859" t="n">
@@ -21282,7 +21282,7 @@
       </c>
       <c r="B860" t="inlineStr">
         <is>
-          <t>And Muhammad Usman Akram</t>
+          <t>Arslan Shaukat</t>
         </is>
       </c>
       <c r="C860" t="n">
@@ -21303,7 +21303,7 @@
       </c>
       <c r="B861" t="inlineStr">
         <is>
-          <t>Mohammed Ghazal</t>
+          <t>Muhammad Owais</t>
         </is>
       </c>
       <c r="C861" t="n">
@@ -21345,7 +21345,7 @@
       </c>
       <c r="B863" t="inlineStr">
         <is>
-          <t>Muhammad Owais</t>
+          <t>Mohammed Ghazal</t>
         </is>
       </c>
       <c r="C863" t="n">

</xml_diff>